<commit_message>
Add: 41.48 MT gitti/concrete (21-Jul) — ₹95,400 material + ₹200 labour = ₹95,600; Papa ₹5K + Self ₹90.6K
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q548"/>
+  <dimension ref="A1:Q550"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23081,33 +23081,153 @@
       </c>
     </row>
     <row r="548">
-      <c r="A548" s="60" t="inlineStr">
+      <c r="A548" t="n">
+        <v>542</v>
+      </c>
+      <c r="B548" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C548">
+        <f>IF(B548="","",TEXT(B548,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>Concrete/Gitti</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>Gitti/Concrete 41.48 MT @ ₹2,300/MT</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="I548" t="n">
+        <v>41.48</v>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="K548" t="n">
+        <v>2300</v>
+      </c>
+      <c r="L548">
+        <f>I548*K548</f>
+        <v/>
+      </c>
+      <c r="N548">
+        <f>M548*L548</f>
+        <v/>
+      </c>
+      <c r="O548">
+        <f>IF(L548="","",IF(M548="",L548,L548*(1-M548)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="n">
+        <v>543</v>
+      </c>
+      <c r="B549" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C549">
+        <f>IF(B549="","",TEXT(B549,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>Labour for gitti/concrete loading</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="I549" t="n">
+        <v>1</v>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K549" t="n">
+        <v>200</v>
+      </c>
+      <c r="L549">
+        <f>I549*K549</f>
+        <v/>
+      </c>
+      <c r="N549">
+        <f>M549*L549</f>
+        <v/>
+      </c>
+      <c r="O549">
+        <f>IF(L549="","",IF(M549="",L549,L549*(1-M549)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B548" s="60" t="n"/>
-      <c r="C548" s="60" t="n"/>
-      <c r="D548" s="60" t="n"/>
-      <c r="E548" s="60" t="n"/>
-      <c r="F548" s="60" t="n"/>
-      <c r="G548" s="60" t="n"/>
-      <c r="H548" s="60" t="n"/>
-      <c r="I548" s="60" t="n"/>
-      <c r="J548" s="60" t="n"/>
-      <c r="K548" s="60" t="n"/>
-      <c r="L548" s="61">
-        <f>SUM(L5:L547)</f>
-        <v/>
-      </c>
-      <c r="M548" s="60" t="n"/>
-      <c r="N548" s="60" t="n"/>
-      <c r="O548" s="61">
+      <c r="B550" s="60" t="n"/>
+      <c r="C550" s="60" t="n"/>
+      <c r="D550" s="60" t="n"/>
+      <c r="E550" s="60" t="n"/>
+      <c r="F550" s="60" t="n"/>
+      <c r="G550" s="60" t="n"/>
+      <c r="H550" s="60" t="n"/>
+      <c r="I550" s="60" t="n"/>
+      <c r="J550" s="60" t="n"/>
+      <c r="K550" s="60" t="n"/>
+      <c r="L550" s="61">
+        <f>SUM(L5:L549)</f>
+        <v/>
+      </c>
+      <c r="M550" s="60" t="n"/>
+      <c r="N550" s="60" t="n"/>
+      <c r="O550" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P548" s="60" t="n"/>
-      <c r="Q548" s="60" t="n"/>
+      <c r="P550" s="60" t="n"/>
+      <c r="Q550" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -37197,32 +37317,92 @@
       <c r="M49" s="47" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="99">
-      <c r="A50" s="43" t="n"/>
-      <c r="B50" s="53" t="n"/>
-      <c r="C50" s="55" t="n"/>
-      <c r="D50" s="55" t="n"/>
-      <c r="E50" s="55" t="n"/>
-      <c r="F50" s="55" t="n"/>
-      <c r="G50" s="63" t="n"/>
-      <c r="H50" s="55" t="n"/>
+      <c r="A50" s="43" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="53" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C50" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D50" s="55" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="E50" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F50" s="55" t="inlineStr">
+        <is>
+          <t>Gitti/Concrete 41.48 MT + labour</t>
+        </is>
+      </c>
+      <c r="G50" s="63" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H50" s="55" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I50" s="55" t="n"/>
       <c r="J50" s="55" t="n"/>
-      <c r="K50" s="55" t="n"/>
+      <c r="K50" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L50" s="58" t="n"/>
       <c r="M50" s="55" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="99">
-      <c r="A51" s="41" t="n"/>
-      <c r="B51" s="45" t="n"/>
-      <c r="C51" s="47" t="n"/>
-      <c r="D51" s="47" t="n"/>
-      <c r="E51" s="47" t="n"/>
-      <c r="F51" s="47" t="n"/>
-      <c r="G51" s="62" t="n"/>
-      <c r="H51" s="47" t="n"/>
+      <c r="A51" s="41" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="45" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C51" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D51" s="47" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="E51" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F51" s="47" t="inlineStr">
+        <is>
+          <t>Gitti/Concrete 41.48 MT + labour</t>
+        </is>
+      </c>
+      <c r="G51" s="62" t="n">
+        <v>90600</v>
+      </c>
+      <c r="H51" s="47" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
       <c r="I51" s="47" t="n"/>
       <c r="J51" s="47" t="n"/>
-      <c r="K51" s="47" t="n"/>
+      <c r="K51" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L51" s="50" t="n"/>
       <c r="M51" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix: Add ₹4 final settlement to Concrete Supplier (Self, 22-Jul)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -37407,17 +37407,47 @@
       <c r="M51" s="47" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="99">
-      <c r="A52" s="43" t="n"/>
-      <c r="B52" s="53" t="n"/>
-      <c r="C52" s="55" t="n"/>
-      <c r="D52" s="55" t="n"/>
-      <c r="E52" s="55" t="n"/>
-      <c r="F52" s="55" t="n"/>
-      <c r="G52" s="63" t="n"/>
-      <c r="H52" s="55" t="n"/>
+      <c r="A52" s="43" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="53" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C52" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D52" s="55" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="E52" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F52" s="55" t="inlineStr">
+        <is>
+          <t>Gitti/Concrete final settlement balance</t>
+        </is>
+      </c>
+      <c r="G52" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="H52" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I52" s="55" t="n"/>
       <c r="J52" s="55" t="n"/>
-      <c r="K52" s="55" t="n"/>
+      <c r="K52" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L52" s="58" t="n"/>
       <c r="M52" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: ₹37,700 Econ Builder supervision fee (21-Jul) + Papa payment
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q550"/>
+  <dimension ref="A1:Q551"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23201,33 +23201,93 @@
       </c>
     </row>
     <row r="550">
-      <c r="A550" s="60" t="inlineStr">
+      <c r="A550" t="n">
+        <v>544</v>
+      </c>
+      <c r="B550" s="128" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C550">
+        <f>IF(B550="","",TEXT(B550,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>Engineer supervision and site coordination</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I550" t="n">
+        <v>1</v>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K550" t="n">
+        <v>37700</v>
+      </c>
+      <c r="L550">
+        <f>I550*K550</f>
+        <v/>
+      </c>
+      <c r="N550">
+        <f>M550*L550</f>
+        <v/>
+      </c>
+      <c r="O550">
+        <f>IF(L550="","",IF(M550="",L550,L550*(1-M550)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B550" s="60" t="n"/>
-      <c r="C550" s="60" t="n"/>
-      <c r="D550" s="60" t="n"/>
-      <c r="E550" s="60" t="n"/>
-      <c r="F550" s="60" t="n"/>
-      <c r="G550" s="60" t="n"/>
-      <c r="H550" s="60" t="n"/>
-      <c r="I550" s="60" t="n"/>
-      <c r="J550" s="60" t="n"/>
-      <c r="K550" s="60" t="n"/>
-      <c r="L550" s="61">
-        <f>SUM(L5:L549)</f>
-        <v/>
-      </c>
-      <c r="M550" s="60" t="n"/>
-      <c r="N550" s="60" t="n"/>
-      <c r="O550" s="61">
+      <c r="B551" s="60" t="n"/>
+      <c r="C551" s="60" t="n"/>
+      <c r="D551" s="60" t="n"/>
+      <c r="E551" s="60" t="n"/>
+      <c r="F551" s="60" t="n"/>
+      <c r="G551" s="60" t="n"/>
+      <c r="H551" s="60" t="n"/>
+      <c r="I551" s="60" t="n"/>
+      <c r="J551" s="60" t="n"/>
+      <c r="K551" s="60" t="n"/>
+      <c r="L551" s="61">
+        <f>SUM(L5:L550)</f>
+        <v/>
+      </c>
+      <c r="M551" s="60" t="n"/>
+      <c r="N551" s="60" t="n"/>
+      <c r="O551" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P550" s="60" t="n"/>
-      <c r="Q550" s="60" t="n"/>
+      <c r="P551" s="60" t="n"/>
+      <c r="Q551" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -37452,17 +37512,47 @@
       <c r="M52" s="55" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="99">
-      <c r="A53" s="41" t="n"/>
-      <c r="B53" s="45" t="n"/>
-      <c r="C53" s="47" t="n"/>
-      <c r="D53" s="47" t="n"/>
-      <c r="E53" s="47" t="n"/>
-      <c r="F53" s="47" t="n"/>
-      <c r="G53" s="62" t="n"/>
-      <c r="H53" s="47" t="n"/>
+      <c r="A53" s="41" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="45" t="n">
+        <v>46224</v>
+      </c>
+      <c r="C53" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D53" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E53" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F53" s="47" t="inlineStr">
+        <is>
+          <t>Engineer supervision and coordination</t>
+        </is>
+      </c>
+      <c r="G53" s="62" t="n">
+        <v>37700</v>
+      </c>
+      <c r="H53" s="47" t="inlineStr">
+        <is>
+          <t>GPay</t>
+        </is>
+      </c>
       <c r="I53" s="47" t="n"/>
       <c r="J53" s="47" t="n"/>
-      <c r="K53" s="47" t="n"/>
+      <c r="K53" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L53" s="50" t="n"/>
       <c r="M53" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: Pappu Hardware cement (22-Jul) — Ultratech Premium 20 bags @ ₹330 + ₹400 labour = ₹7,000 (Self, Cash)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q551"/>
+  <dimension ref="A1:Q553"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23261,33 +23261,153 @@
       </c>
     </row>
     <row r="551">
-      <c r="A551" s="60" t="inlineStr">
+      <c r="A551" t="n">
+        <v>545</v>
+      </c>
+      <c r="B551" s="128" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C551">
+        <f>IF(B551="","",TEXT(B551,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>Ultratech Premium Cement 20 bags @ ₹330</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I551" t="n">
+        <v>20</v>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K551" t="n">
+        <v>330</v>
+      </c>
+      <c r="L551">
+        <f>I551*K551</f>
+        <v/>
+      </c>
+      <c r="N551">
+        <f>M551*L551</f>
+        <v/>
+      </c>
+      <c r="O551">
+        <f>IF(L551="","",IF(M551="",L551,L551*(1-M551)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>546</v>
+      </c>
+      <c r="B552" s="128" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C552">
+        <f>IF(B552="","",TEXT(B552,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>Labour for cement handling/loading</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I552" t="n">
+        <v>1</v>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K552" t="n">
+        <v>400</v>
+      </c>
+      <c r="L552">
+        <f>I552*K552</f>
+        <v/>
+      </c>
+      <c r="N552">
+        <f>M552*L552</f>
+        <v/>
+      </c>
+      <c r="O552">
+        <f>IF(L552="","",IF(M552="",L552,L552*(1-M552)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B551" s="60" t="n"/>
-      <c r="C551" s="60" t="n"/>
-      <c r="D551" s="60" t="n"/>
-      <c r="E551" s="60" t="n"/>
-      <c r="F551" s="60" t="n"/>
-      <c r="G551" s="60" t="n"/>
-      <c r="H551" s="60" t="n"/>
-      <c r="I551" s="60" t="n"/>
-      <c r="J551" s="60" t="n"/>
-      <c r="K551" s="60" t="n"/>
-      <c r="L551" s="61">
-        <f>SUM(L5:L550)</f>
-        <v/>
-      </c>
-      <c r="M551" s="60" t="n"/>
-      <c r="N551" s="60" t="n"/>
-      <c r="O551" s="61">
+      <c r="B553" s="60" t="n"/>
+      <c r="C553" s="60" t="n"/>
+      <c r="D553" s="60" t="n"/>
+      <c r="E553" s="60" t="n"/>
+      <c r="F553" s="60" t="n"/>
+      <c r="G553" s="60" t="n"/>
+      <c r="H553" s="60" t="n"/>
+      <c r="I553" s="60" t="n"/>
+      <c r="J553" s="60" t="n"/>
+      <c r="K553" s="60" t="n"/>
+      <c r="L553" s="61">
+        <f>SUM(L5:L552)</f>
+        <v/>
+      </c>
+      <c r="M553" s="60" t="n"/>
+      <c r="N553" s="60" t="n"/>
+      <c r="O553" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P551" s="60" t="n"/>
-      <c r="Q551" s="60" t="n"/>
+      <c r="P553" s="60" t="n"/>
+      <c r="Q553" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -37557,17 +37677,47 @@
       <c r="M53" s="47" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="99">
-      <c r="A54" s="43" t="n"/>
-      <c r="B54" s="53" t="n"/>
-      <c r="C54" s="55" t="n"/>
-      <c r="D54" s="55" t="n"/>
-      <c r="E54" s="55" t="n"/>
-      <c r="F54" s="55" t="n"/>
-      <c r="G54" s="63" t="n"/>
-      <c r="H54" s="55" t="n"/>
+      <c r="A54" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="53" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C54" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D54" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E54" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials + Labour</t>
+        </is>
+      </c>
+      <c r="F54" s="55" t="inlineStr">
+        <is>
+          <t>Cement 20 bags + labour</t>
+        </is>
+      </c>
+      <c r="G54" s="63" t="n">
+        <v>7000</v>
+      </c>
+      <c r="H54" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I54" s="55" t="n"/>
       <c r="J54" s="55" t="n"/>
-      <c r="K54" s="55" t="n"/>
+      <c r="K54" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L54" s="58" t="n"/>
       <c r="M54" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: ₹4,000 Econ Builder (Papa, 31-Jul) — Santosh aara mil (payment received, Cash)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q553"/>
+  <dimension ref="A1:Q554"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23381,33 +23381,93 @@
       </c>
     </row>
     <row r="553">
-      <c r="A553" s="60" t="inlineStr">
+      <c r="A553" t="n">
+        <v>547</v>
+      </c>
+      <c r="B553" s="128" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C553">
+        <f>IF(B553="","",TEXT(B553,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>Payment to Santosh — aara mil (received)</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I553" t="n">
+        <v>1</v>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K553" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L553">
+        <f>I553*K553</f>
+        <v/>
+      </c>
+      <c r="N553">
+        <f>M553*L553</f>
+        <v/>
+      </c>
+      <c r="O553">
+        <f>IF(L553="","",IF(M553="",L553,L553*(1-M553)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B553" s="60" t="n"/>
-      <c r="C553" s="60" t="n"/>
-      <c r="D553" s="60" t="n"/>
-      <c r="E553" s="60" t="n"/>
-      <c r="F553" s="60" t="n"/>
-      <c r="G553" s="60" t="n"/>
-      <c r="H553" s="60" t="n"/>
-      <c r="I553" s="60" t="n"/>
-      <c r="J553" s="60" t="n"/>
-      <c r="K553" s="60" t="n"/>
-      <c r="L553" s="61">
-        <f>SUM(L5:L552)</f>
-        <v/>
-      </c>
-      <c r="M553" s="60" t="n"/>
-      <c r="N553" s="60" t="n"/>
-      <c r="O553" s="61">
+      <c r="B554" s="60" t="n"/>
+      <c r="C554" s="60" t="n"/>
+      <c r="D554" s="60" t="n"/>
+      <c r="E554" s="60" t="n"/>
+      <c r="F554" s="60" t="n"/>
+      <c r="G554" s="60" t="n"/>
+      <c r="H554" s="60" t="n"/>
+      <c r="I554" s="60" t="n"/>
+      <c r="J554" s="60" t="n"/>
+      <c r="K554" s="60" t="n"/>
+      <c r="L554" s="61">
+        <f>SUM(L5:L553)</f>
+        <v/>
+      </c>
+      <c r="M554" s="60" t="n"/>
+      <c r="N554" s="60" t="n"/>
+      <c r="O554" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P553" s="60" t="n"/>
-      <c r="Q553" s="60" t="n"/>
+      <c r="P554" s="60" t="n"/>
+      <c r="Q554" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -37722,17 +37782,47 @@
       <c r="M54" s="55" t="n"/>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="99">
-      <c r="A55" s="41" t="n"/>
-      <c r="B55" s="45" t="n"/>
-      <c r="C55" s="47" t="n"/>
-      <c r="D55" s="47" t="n"/>
-      <c r="E55" s="47" t="n"/>
-      <c r="F55" s="47" t="n"/>
-      <c r="G55" s="62" t="n"/>
-      <c r="H55" s="47" t="n"/>
+      <c r="A55" s="41" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="45" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C55" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D55" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E55" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F55" s="47" t="inlineStr">
+        <is>
+          <t>Santosh aara mil — payment received</t>
+        </is>
+      </c>
+      <c r="G55" s="62" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H55" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I55" s="47" t="n"/>
       <c r="J55" s="47" t="n"/>
-      <c r="K55" s="47" t="n"/>
+      <c r="K55" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L55" s="50" t="n"/>
       <c r="M55" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
FINAL: ₹32,950 Mukesh Yadav settlement (2-Aug) — ALL VENDORS SETTLED, Project financially closed
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -37827,17 +37827,47 @@
       <c r="M55" s="47" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="99">
-      <c r="A56" s="43" t="n"/>
-      <c r="B56" s="53" t="n"/>
-      <c r="C56" s="55" t="n"/>
-      <c r="D56" s="55" t="n"/>
-      <c r="E56" s="55" t="n"/>
-      <c r="F56" s="55" t="n"/>
-      <c r="G56" s="63" t="n"/>
-      <c r="H56" s="55" t="n"/>
+      <c r="A56" s="43" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="53" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C56" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D56" s="55" t="inlineStr">
+        <is>
+          <t>Mukesh Yadav</t>
+        </is>
+      </c>
+      <c r="E56" s="55" t="inlineStr">
+        <is>
+          <t>Land Development + Labour</t>
+        </is>
+      </c>
+      <c r="F56" s="55" t="inlineStr">
+        <is>
+          <t>JCB + Mitti + Sand movement — final settlement</t>
+        </is>
+      </c>
+      <c r="G56" s="63" t="n">
+        <v>32950</v>
+      </c>
+      <c r="H56" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I56" s="55" t="n"/>
       <c r="J56" s="55" t="n"/>
-      <c r="K56" s="55" t="n"/>
+      <c r="K56" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L56" s="58" t="n"/>
       <c r="M56" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: Pappu Hardware ₹47,740 (7-Aug) — cement, 10mm/6mm rod, wire, labour
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q554"/>
+  <dimension ref="A1:Q559"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23441,33 +23441,333 @@
       </c>
     </row>
     <row r="554">
-      <c r="A554" s="60" t="inlineStr">
+      <c r="A554" t="n">
+        <v>548</v>
+      </c>
+      <c r="B554" s="128" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C554">
+        <f>IF(B554="","",TEXT(B554,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>Ultratech Super cement 25 bags @ ₹350</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I554" t="n">
+        <v>25</v>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K554" t="n">
+        <v>350</v>
+      </c>
+      <c r="L554">
+        <f>I554*K554</f>
+        <v/>
+      </c>
+      <c r="N554">
+        <f>M554*L554</f>
+        <v/>
+      </c>
+      <c r="O554">
+        <f>IF(L554="","",IF(M554="",L554,L554*(1-M554)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>549</v>
+      </c>
+      <c r="B555" s="128" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C555">
+        <f>IF(B555="","",TEXT(B555,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>10mm Tata Tiscon Rod 50 pcs @ ₹590 (4% disc)</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I555" t="n">
+        <v>50</v>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K555" t="n">
+        <v>566.4</v>
+      </c>
+      <c r="L555">
+        <f>I555*K555</f>
+        <v/>
+      </c>
+      <c r="N555">
+        <f>M555*L555</f>
+        <v/>
+      </c>
+      <c r="O555">
+        <f>IF(L555="","",IF(M555="",L555,L555*(1-M555)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>550</v>
+      </c>
+      <c r="B556" s="128" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C556">
+        <f>IF(B556="","",TEXT(B556,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>6mm Tata Tiscon Rod 40 pcs @ ₹228</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I556" t="n">
+        <v>40</v>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K556" t="n">
+        <v>228</v>
+      </c>
+      <c r="L556">
+        <f>I556*K556</f>
+        <v/>
+      </c>
+      <c r="N556">
+        <f>M556*L556</f>
+        <v/>
+      </c>
+      <c r="O556">
+        <f>IF(L556="","",IF(M556="",L556,L556*(1-M556)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>551</v>
+      </c>
+      <c r="B557" s="128" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C557">
+        <f>IF(B557="","",TEXT(B557,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>Tata soft wire 10 Kg @ ₹110</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I557" t="n">
+        <v>10</v>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="K557" t="n">
+        <v>110</v>
+      </c>
+      <c r="L557">
+        <f>I557*K557</f>
+        <v/>
+      </c>
+      <c r="N557">
+        <f>M557*L557</f>
+        <v/>
+      </c>
+      <c r="O557">
+        <f>IF(L557="","",IF(M557="",L557,L557*(1-M557)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>552</v>
+      </c>
+      <c r="B558" s="128" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C558">
+        <f>IF(B558="","",TEXT(B558,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>Labour for loading/handling</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I558" t="n">
+        <v>1</v>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K558" t="n">
+        <v>450</v>
+      </c>
+      <c r="L558">
+        <f>I558*K558</f>
+        <v/>
+      </c>
+      <c r="N558">
+        <f>M558*L558</f>
+        <v/>
+      </c>
+      <c r="O558">
+        <f>IF(L558="","",IF(M558="",L558,L558*(1-M558)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B554" s="60" t="n"/>
-      <c r="C554" s="60" t="n"/>
-      <c r="D554" s="60" t="n"/>
-      <c r="E554" s="60" t="n"/>
-      <c r="F554" s="60" t="n"/>
-      <c r="G554" s="60" t="n"/>
-      <c r="H554" s="60" t="n"/>
-      <c r="I554" s="60" t="n"/>
-      <c r="J554" s="60" t="n"/>
-      <c r="K554" s="60" t="n"/>
-      <c r="L554" s="61">
-        <f>SUM(L5:L553)</f>
-        <v/>
-      </c>
-      <c r="M554" s="60" t="n"/>
-      <c r="N554" s="60" t="n"/>
-      <c r="O554" s="61">
+      <c r="B559" s="60" t="n"/>
+      <c r="C559" s="60" t="n"/>
+      <c r="D559" s="60" t="n"/>
+      <c r="E559" s="60" t="n"/>
+      <c r="F559" s="60" t="n"/>
+      <c r="G559" s="60" t="n"/>
+      <c r="H559" s="60" t="n"/>
+      <c r="I559" s="60" t="n"/>
+      <c r="J559" s="60" t="n"/>
+      <c r="K559" s="60" t="n"/>
+      <c r="L559" s="61">
+        <f>SUM(L5:L558)</f>
+        <v/>
+      </c>
+      <c r="M559" s="60" t="n"/>
+      <c r="N559" s="60" t="n"/>
+      <c r="O559" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P554" s="60" t="n"/>
-      <c r="Q554" s="60" t="n"/>
+      <c r="P559" s="60" t="n"/>
+      <c r="Q559" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -37872,17 +38172,47 @@
       <c r="M56" s="55" t="n"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="99">
-      <c r="A57" s="41" t="n"/>
-      <c r="B57" s="45" t="n"/>
-      <c r="C57" s="47" t="n"/>
-      <c r="D57" s="47" t="n"/>
-      <c r="E57" s="47" t="n"/>
-      <c r="F57" s="47" t="n"/>
-      <c r="G57" s="62" t="n"/>
-      <c r="H57" s="47" t="n"/>
+      <c r="A57" s="41" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="45" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C57" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D57" s="47" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E57" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials + Steel + Labour</t>
+        </is>
+      </c>
+      <c r="F57" s="47" t="inlineStr">
+        <is>
+          <t>Cement + Tata Tiscon rods + wire + labour</t>
+        </is>
+      </c>
+      <c r="G57" s="62" t="n">
+        <v>47740</v>
+      </c>
+      <c r="H57" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I57" s="47" t="n"/>
       <c r="J57" s="47" t="n"/>
-      <c r="K57" s="47" t="n"/>
+      <c r="K57" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L57" s="50" t="n"/>
       <c r="M57" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: ₹37,900 Econ Builder (Papa, 9-Aug) — Darbhanga labour, chotu lohabala, grilling, 4mm ply, Bayju
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q559"/>
+  <dimension ref="A1:Q564"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -23741,33 +23741,333 @@
       </c>
     </row>
     <row r="559">
-      <c r="A559" s="60" t="inlineStr">
+      <c r="A559" t="n">
+        <v>553</v>
+      </c>
+      <c r="B559" s="128" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C559">
+        <f>IF(B559="","",TEXT(B559,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>Darbhanga labour payment</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I559" t="n">
+        <v>1</v>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="K559" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L559">
+        <f>I559*K559</f>
+        <v/>
+      </c>
+      <c r="N559">
+        <f>M559*L559</f>
+        <v/>
+      </c>
+      <c r="O559">
+        <f>IF(L559="","",IF(M559="",L559,L559*(1-M559)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>554</v>
+      </c>
+      <c r="B560" s="128" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C560">
+        <f>IF(B560="","",TEXT(B560,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Fabrication</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>Chotu lohabala</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I560" t="n">
+        <v>1</v>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="K560" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L560">
+        <f>I560*K560</f>
+        <v/>
+      </c>
+      <c r="N560">
+        <f>M560*L560</f>
+        <v/>
+      </c>
+      <c r="O560">
+        <f>IF(L560="","",IF(M560="",L560,L560*(1-M560)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>555</v>
+      </c>
+      <c r="B561" s="128" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C561">
+        <f>IF(B561="","",TEXT(B561,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Fabrication</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Grilling</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I561" t="n">
+        <v>1</v>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K561" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L561">
+        <f>I561*K561</f>
+        <v/>
+      </c>
+      <c r="N561">
+        <f>M561*L561</f>
+        <v/>
+      </c>
+      <c r="O561">
+        <f>IF(L561="","",IF(M561="",L561,L561*(1-M561)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>556</v>
+      </c>
+      <c r="B562" s="128" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C562">
+        <f>IF(B562="","",TEXT(B562,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Plywood/Shuttering</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>4mm ply</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I562" t="n">
+        <v>1</v>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="K562" t="n">
+        <v>700</v>
+      </c>
+      <c r="L562">
+        <f>I562*K562</f>
+        <v/>
+      </c>
+      <c r="N562">
+        <f>M562*L562</f>
+        <v/>
+      </c>
+      <c r="O562">
+        <f>IF(L562="","",IF(M562="",L562,L562*(1-M562)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>557</v>
+      </c>
+      <c r="B563" s="128" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C563">
+        <f>IF(B563="","",TEXT(B563,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Bayju</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I563" t="n">
+        <v>1</v>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="K563" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L563">
+        <f>I563*K563</f>
+        <v/>
+      </c>
+      <c r="N563">
+        <f>M563*L563</f>
+        <v/>
+      </c>
+      <c r="O563">
+        <f>IF(L563="","",IF(M563="",L563,L563*(1-M563)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B559" s="60" t="n"/>
-      <c r="C559" s="60" t="n"/>
-      <c r="D559" s="60" t="n"/>
-      <c r="E559" s="60" t="n"/>
-      <c r="F559" s="60" t="n"/>
-      <c r="G559" s="60" t="n"/>
-      <c r="H559" s="60" t="n"/>
-      <c r="I559" s="60" t="n"/>
-      <c r="J559" s="60" t="n"/>
-      <c r="K559" s="60" t="n"/>
-      <c r="L559" s="61">
-        <f>SUM(L5:L558)</f>
-        <v/>
-      </c>
-      <c r="M559" s="60" t="n"/>
-      <c r="N559" s="60" t="n"/>
-      <c r="O559" s="61">
+      <c r="B564" s="60" t="n"/>
+      <c r="C564" s="60" t="n"/>
+      <c r="D564" s="60" t="n"/>
+      <c r="E564" s="60" t="n"/>
+      <c r="F564" s="60" t="n"/>
+      <c r="G564" s="60" t="n"/>
+      <c r="H564" s="60" t="n"/>
+      <c r="I564" s="60" t="n"/>
+      <c r="J564" s="60" t="n"/>
+      <c r="K564" s="60" t="n"/>
+      <c r="L564" s="61">
+        <f>SUM(L5:L563)</f>
+        <v/>
+      </c>
+      <c r="M564" s="60" t="n"/>
+      <c r="N564" s="60" t="n"/>
+      <c r="O564" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P559" s="60" t="n"/>
-      <c r="Q559" s="60" t="n"/>
+      <c r="P564" s="60" t="n"/>
+      <c r="Q564" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -35716,7 +36016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M504"/>
+  <dimension ref="A1:M505"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -38217,17 +38517,47 @@
       <c r="M57" s="47" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="99">
-      <c r="A58" s="43" t="n"/>
-      <c r="B58" s="53" t="n"/>
-      <c r="C58" s="55" t="n"/>
-      <c r="D58" s="55" t="n"/>
-      <c r="E58" s="55" t="n"/>
-      <c r="F58" s="55" t="n"/>
-      <c r="G58" s="63" t="n"/>
-      <c r="H58" s="55" t="n"/>
+      <c r="A58" s="43" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="53" t="n">
+        <v>46243</v>
+      </c>
+      <c r="C58" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D58" s="55" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E58" s="55" t="inlineStr">
+        <is>
+          <t>Labour + Steel/Iron + Building Materials</t>
+        </is>
+      </c>
+      <c r="F58" s="55" t="inlineStr">
+        <is>
+          <t>Darbhanga labour, chotu lohabala, grilling, 4mm ply, Bayju</t>
+        </is>
+      </c>
+      <c r="G58" s="63" t="n">
+        <v>37900</v>
+      </c>
+      <c r="H58" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I58" s="55" t="n"/>
       <c r="J58" s="55" t="n"/>
-      <c r="K58" s="55" t="n"/>
+      <c r="K58" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L58" s="58" t="n"/>
       <c r="M58" s="55" t="n"/>
     </row>
@@ -46945,6 +47275,14 @@
         <v/>
       </c>
       <c r="M504" s="55" t="n"/>
+    </row>
+    <row r="505">
+      <c r="B505" s="128" t="n"/>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M504"/>

</xml_diff>

<commit_message>
Add: 7 more brick trailers (22-Aug) — 10,500 bricks, tractor 21-27 @ ₹8.5
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q564"/>
+  <dimension ref="A1:Q565"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -24041,33 +24041,93 @@
       </c>
     </row>
     <row r="564">
-      <c r="A564" s="60" t="inlineStr">
+      <c r="A564" t="n">
+        <v>558</v>
+      </c>
+      <c r="B564" s="128" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C564">
+        <f>IF(B564="","",TEXT(B564,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>Brick delivery — tractor 21-27 (10,500 bricks @ ₹8.5)</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Brick Company</t>
+        </is>
+      </c>
+      <c r="I564" t="n">
+        <v>10500</v>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K564" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L564">
+        <f>I564*K564</f>
+        <v/>
+      </c>
+      <c r="N564">
+        <f>M564*L564</f>
+        <v/>
+      </c>
+      <c r="O564">
+        <f>IF(L564="","",IF(M564="",L564,L564*(1-M564)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B564" s="60" t="n"/>
-      <c r="C564" s="60" t="n"/>
-      <c r="D564" s="60" t="n"/>
-      <c r="E564" s="60" t="n"/>
-      <c r="F564" s="60" t="n"/>
-      <c r="G564" s="60" t="n"/>
-      <c r="H564" s="60" t="n"/>
-      <c r="I564" s="60" t="n"/>
-      <c r="J564" s="60" t="n"/>
-      <c r="K564" s="60" t="n"/>
-      <c r="L564" s="61">
-        <f>SUM(L5:L563)</f>
-        <v/>
-      </c>
-      <c r="M564" s="60" t="n"/>
-      <c r="N564" s="60" t="n"/>
-      <c r="O564" s="61">
+      <c r="B565" s="60" t="n"/>
+      <c r="C565" s="60" t="n"/>
+      <c r="D565" s="60" t="n"/>
+      <c r="E565" s="60" t="n"/>
+      <c r="F565" s="60" t="n"/>
+      <c r="G565" s="60" t="n"/>
+      <c r="H565" s="60" t="n"/>
+      <c r="I565" s="60" t="n"/>
+      <c r="J565" s="60" t="n"/>
+      <c r="K565" s="60" t="n"/>
+      <c r="L565" s="61">
+        <f>SUM(L5:L564)</f>
+        <v/>
+      </c>
+      <c r="M565" s="60" t="n"/>
+      <c r="N565" s="60" t="n"/>
+      <c r="O565" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P564" s="60" t="n"/>
-      <c r="Q564" s="60" t="n"/>
+      <c r="P565" s="60" t="n"/>
+      <c r="Q565" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>

<commit_message>
Add: ₹17,100 Pappu Hardware (Avinash, 24-Aug) — Ultratech Super+Plain cement, labour
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6453,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q565"/>
+  <dimension ref="A1:Q568"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -24101,33 +24101,213 @@
       </c>
     </row>
     <row r="565">
-      <c r="A565" s="60" t="inlineStr">
+      <c r="A565" t="n">
+        <v>559</v>
+      </c>
+      <c r="B565" s="128" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C565">
+        <f>IF(B565="","",TEXT(B565,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>Ultratech Super cement 30 bags @ ₹340</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I565" t="n">
+        <v>30</v>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K565" t="n">
+        <v>340</v>
+      </c>
+      <c r="L565">
+        <f>I565*K565</f>
+        <v/>
+      </c>
+      <c r="N565">
+        <f>M565*L565</f>
+        <v/>
+      </c>
+      <c r="O565">
+        <f>IF(L565="","",IF(M565="",L565,L565*(1-M565)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="n">
+        <v>560</v>
+      </c>
+      <c r="B566" s="128" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C566">
+        <f>IF(B566="","",TEXT(B566,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>Ultratech Plain cement 20 bags @ ₹320</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I566" t="n">
+        <v>20</v>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K566" t="n">
+        <v>320</v>
+      </c>
+      <c r="L566">
+        <f>I566*K566</f>
+        <v/>
+      </c>
+      <c r="N566">
+        <f>M566*L566</f>
+        <v/>
+      </c>
+      <c r="O566">
+        <f>IF(L566="","",IF(M566="",L566,L566*(1-M566)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="n">
+        <v>561</v>
+      </c>
+      <c r="B567" s="128" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C567">
+        <f>IF(B567="","",TEXT(B567,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I567" t="n">
+        <v>1</v>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K567" t="n">
+        <v>500</v>
+      </c>
+      <c r="L567">
+        <f>I567*K567</f>
+        <v/>
+      </c>
+      <c r="N567">
+        <f>M567*L567</f>
+        <v/>
+      </c>
+      <c r="O567">
+        <f>IF(L567="","",IF(M567="",L567,L567*(1-M567)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B565" s="60" t="n"/>
-      <c r="C565" s="60" t="n"/>
-      <c r="D565" s="60" t="n"/>
-      <c r="E565" s="60" t="n"/>
-      <c r="F565" s="60" t="n"/>
-      <c r="G565" s="60" t="n"/>
-      <c r="H565" s="60" t="n"/>
-      <c r="I565" s="60" t="n"/>
-      <c r="J565" s="60" t="n"/>
-      <c r="K565" s="60" t="n"/>
-      <c r="L565" s="61">
-        <f>SUM(L5:L564)</f>
-        <v/>
-      </c>
-      <c r="M565" s="60" t="n"/>
-      <c r="N565" s="60" t="n"/>
-      <c r="O565" s="61">
+      <c r="B568" s="60" t="n"/>
+      <c r="C568" s="60" t="n"/>
+      <c r="D568" s="60" t="n"/>
+      <c r="E568" s="60" t="n"/>
+      <c r="F568" s="60" t="n"/>
+      <c r="G568" s="60" t="n"/>
+      <c r="H568" s="60" t="n"/>
+      <c r="I568" s="60" t="n"/>
+      <c r="J568" s="60" t="n"/>
+      <c r="K568" s="60" t="n"/>
+      <c r="L568" s="61">
+        <f>SUM(L5:L567)</f>
+        <v/>
+      </c>
+      <c r="M568" s="60" t="n"/>
+      <c r="N568" s="60" t="n"/>
+      <c r="O568" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P565" s="60" t="n"/>
-      <c r="Q565" s="60" t="n"/>
+      <c r="P568" s="60" t="n"/>
+      <c r="Q568" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -38622,17 +38802,47 @@
       <c r="M58" s="55" t="n"/>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="99">
-      <c r="A59" s="41" t="n"/>
-      <c r="B59" s="45" t="n"/>
-      <c r="C59" s="47" t="n"/>
-      <c r="D59" s="47" t="n"/>
-      <c r="E59" s="47" t="n"/>
-      <c r="F59" s="47" t="n"/>
-      <c r="G59" s="62" t="n"/>
-      <c r="H59" s="47" t="n"/>
+      <c r="A59" s="41" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="45" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C59" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D59" s="47" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E59" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials + Labour</t>
+        </is>
+      </c>
+      <c r="F59" s="47" t="inlineStr">
+        <is>
+          <t>Ultratech Super + Plain cement, labour</t>
+        </is>
+      </c>
+      <c r="G59" s="62" t="n">
+        <v>17100</v>
+      </c>
+      <c r="H59" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I59" s="47" t="n"/>
       <c r="J59" s="47" t="n"/>
-      <c r="K59" s="47" t="n"/>
+      <c r="K59" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L59" s="50" t="n"/>
       <c r="M59" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: Unit Funding section — B/C-Unit 50/50 split + Deepu's ₹15L C-Unit fund tracker
- New 'Unit Funding' sheet in Excel: funder, unit, commitment, family-funded threshold
- New optional 'Building Unit' tag column on All Transactions (blank = joint, split 50/50)
- Generator computes B/C spend split and funder utilization/remaining
- New dashboard card: unit split + funder progress (committed/used/remaining)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Labour Tracker" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Monthly Summary" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Vendor Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Unit Funding" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Transactions'!$A$4:$Q$504</definedName>
@@ -2938,6 +2939,91 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="99" min="1" max="1"/>
+    <col width="8" customWidth="1" style="99" min="2" max="2"/>
+    <col width="16" customWidth="1" style="99" min="3" max="3"/>
+    <col width="40" customWidth="1" style="99" min="4" max="4"/>
+    <col width="60" customWidth="1" style="99" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UNIT FUNDING — B-Unit / C-Unit cost split &amp; external funder commitments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All spend is split 50/50 between B-Unit and C-Unit unless a transaction is explicitly tagged to one unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Funder</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Commitment ₹</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Family-funded threshold ₹ (kicks in after this much unit spend)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Deepu</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Avinash funds first ₹10L of C-Unit spend; Deepu funds the next ₹15L of C-Unit spend beyond that</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6453,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q568"/>
+  <dimension ref="A1:R568"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -6472,6 +6558,7 @@
     <col width="14" customWidth="1" style="99" min="15" max="15"/>
     <col width="18" customWidth="1" style="99" min="16" max="16"/>
     <col width="14" customWidth="1" style="99" min="17" max="17"/>
+    <col width="30" customWidth="1" style="99" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="99">
@@ -6572,6 +6659,11 @@
       <c r="Q4" s="40" t="inlineStr">
         <is>
           <t>Payment Mode</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Building Unit (B/C, blank=joint 50/50)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add: 2 more brick trailers (23-Aug) — 3,000 bricks, tractor 28-29 @ ₹8.5
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R568"/>
+  <dimension ref="A1:R569"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -24373,33 +24373,93 @@
       </c>
     </row>
     <row r="568">
-      <c r="A568" s="60" t="inlineStr">
+      <c r="A568" t="n">
+        <v>562</v>
+      </c>
+      <c r="B568" s="128" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C568">
+        <f>IF(B568="","",TEXT(B568,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Brick delivery — tractor 28-29 (3,000 bricks @ ₹8.5)</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>Brick Company</t>
+        </is>
+      </c>
+      <c r="I568" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K568" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L568">
+        <f>I568*K568</f>
+        <v/>
+      </c>
+      <c r="N568">
+        <f>M568*L568</f>
+        <v/>
+      </c>
+      <c r="O568">
+        <f>IF(L568="","",IF(M568="",L568,L568*(1-M568)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B568" s="60" t="n"/>
-      <c r="C568" s="60" t="n"/>
-      <c r="D568" s="60" t="n"/>
-      <c r="E568" s="60" t="n"/>
-      <c r="F568" s="60" t="n"/>
-      <c r="G568" s="60" t="n"/>
-      <c r="H568" s="60" t="n"/>
-      <c r="I568" s="60" t="n"/>
-      <c r="J568" s="60" t="n"/>
-      <c r="K568" s="60" t="n"/>
-      <c r="L568" s="61">
-        <f>SUM(L5:L567)</f>
-        <v/>
-      </c>
-      <c r="M568" s="60" t="n"/>
-      <c r="N568" s="60" t="n"/>
-      <c r="O568" s="61">
+      <c r="B569" s="60" t="n"/>
+      <c r="C569" s="60" t="n"/>
+      <c r="D569" s="60" t="n"/>
+      <c r="E569" s="60" t="n"/>
+      <c r="F569" s="60" t="n"/>
+      <c r="G569" s="60" t="n"/>
+      <c r="H569" s="60" t="n"/>
+      <c r="I569" s="60" t="n"/>
+      <c r="J569" s="60" t="n"/>
+      <c r="K569" s="60" t="n"/>
+      <c r="L569" s="61">
+        <f>SUM(L5:L568)</f>
+        <v/>
+      </c>
+      <c r="M569" s="60" t="n"/>
+      <c r="N569" s="60" t="n"/>
+      <c r="O569" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P568" s="60" t="n"/>
-      <c r="Q568" s="60" t="n"/>
+      <c r="P569" s="60" t="n"/>
+      <c r="Q569" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>

<commit_message>
Fix: normalize 'Cement-Ultratech Super' sub-category to 'Cement' (was splitting Breakdown into two lines)
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6832,7 +6832,7 @@
       </c>
       <c r="F7" s="47" t="inlineStr">
         <is>
-          <t>Cement-Ultratech Super</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="G7" s="47" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
       <c r="F34" s="55" t="inlineStr">
         <is>
-          <t>Cement-Ultratech Super</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="G34" s="55" t="inlineStr">
@@ -9389,7 +9389,7 @@
       </c>
       <c r="F44" s="55" t="inlineStr">
         <is>
-          <t>Cement-Ultratech Super</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="G44" s="55" t="inlineStr">
@@ -10306,7 +10306,7 @@
       </c>
       <c r="F57" s="55" t="inlineStr">
         <is>
-          <t>Cement-Ultratech Super</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="G57" s="55" t="inlineStr">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="F63" s="55" t="inlineStr">
         <is>
-          <t>Cement-Ultratech Super</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="G63" s="55" t="inlineStr">

</xml_diff>

<commit_message>
Add: quantity breakup in Breakdown tab (e.g. Cement · 515 bags, Tiscon 12mm · 200 pcs)
- Generator aggregates qty per sub-category when item-unit is consistent, normalized (bags/pcs/kg/CFT/litres/MT/trailers/hours/trips)
- Skips quantity display when units are mixed/inconsistent, to avoid showing misleading totals
- Fixed 2 Sand Truck entries (5-Jul) that had qty=1/Lumpsum instead of real CFT — now 944 and 936 CFT
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -21287,15 +21287,15 @@
         </is>
       </c>
       <c r="I517" t="n">
-        <v>1</v>
+        <v>944</v>
       </c>
       <c r="J517" t="inlineStr">
         <is>
-          <t>Lumpsum</t>
+          <t>CFT</t>
         </is>
       </c>
       <c r="K517" t="n">
-        <v>56500</v>
+        <v>59.85169491525424</v>
       </c>
       <c r="L517">
         <f>IF(OR(I517="",K517=""),"",I517*K517)</f>
@@ -21343,15 +21343,15 @@
         </is>
       </c>
       <c r="I518" t="n">
-        <v>1</v>
+        <v>936</v>
       </c>
       <c r="J518" t="inlineStr">
         <is>
-          <t>Lumpsum</t>
+          <t>CFT</t>
         </is>
       </c>
       <c r="K518" t="n">
-        <v>56000</v>
+        <v>59.82905982905983</v>
       </c>
       <c r="L518">
         <f>IF(OR(I518="",K518=""),"",I518*K518)</f>

</xml_diff>

<commit_message>
Add: ₹12,210 Pappu Hardware (Avinash, 5-Sep) — Ultratech Super+Plain cement, transport
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R569"/>
+  <dimension ref="A1:R572"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -24433,33 +24433,213 @@
       </c>
     </row>
     <row r="569">
-      <c r="A569" s="60" t="inlineStr">
+      <c r="A569" t="n">
+        <v>563</v>
+      </c>
+      <c r="B569" s="128" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C569">
+        <f>IF(B569="","",TEXT(B569,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Ultratech Super cement 12 bags @ ₹340</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I569" t="n">
+        <v>12</v>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K569" t="n">
+        <v>340</v>
+      </c>
+      <c r="L569">
+        <f>I569*K569</f>
+        <v/>
+      </c>
+      <c r="N569">
+        <f>M569*L569</f>
+        <v/>
+      </c>
+      <c r="O569">
+        <f>IF(L569="","",IF(M569="",L569,L569*(1-M569)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="n">
+        <v>564</v>
+      </c>
+      <c r="B570" s="128" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C570">
+        <f>IF(B570="","",TEXT(B570,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Ultratech Plain cement 24 bags @ ₹320</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I570" t="n">
+        <v>24</v>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K570" t="n">
+        <v>320</v>
+      </c>
+      <c r="L570">
+        <f>I570*K570</f>
+        <v/>
+      </c>
+      <c r="N570">
+        <f>M570*L570</f>
+        <v/>
+      </c>
+      <c r="O570">
+        <f>IF(L570="","",IF(M570="",L570,L570*(1-M570)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="n">
+        <v>565</v>
+      </c>
+      <c r="B571" s="128" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C571">
+        <f>IF(B571="","",TEXT(B571,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Material Transport</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>Cement transportation</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I571" t="n">
+        <v>1</v>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>Trip</t>
+        </is>
+      </c>
+      <c r="K571" t="n">
+        <v>450</v>
+      </c>
+      <c r="L571">
+        <f>I571*K571</f>
+        <v/>
+      </c>
+      <c r="N571">
+        <f>M571*L571</f>
+        <v/>
+      </c>
+      <c r="O571">
+        <f>IF(L571="","",IF(M571="",L571,L571*(1-M571)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B569" s="60" t="n"/>
-      <c r="C569" s="60" t="n"/>
-      <c r="D569" s="60" t="n"/>
-      <c r="E569" s="60" t="n"/>
-      <c r="F569" s="60" t="n"/>
-      <c r="G569" s="60" t="n"/>
-      <c r="H569" s="60" t="n"/>
-      <c r="I569" s="60" t="n"/>
-      <c r="J569" s="60" t="n"/>
-      <c r="K569" s="60" t="n"/>
-      <c r="L569" s="61">
-        <f>SUM(L5:L568)</f>
-        <v/>
-      </c>
-      <c r="M569" s="60" t="n"/>
-      <c r="N569" s="60" t="n"/>
-      <c r="O569" s="61">
+      <c r="B572" s="60" t="n"/>
+      <c r="C572" s="60" t="n"/>
+      <c r="D572" s="60" t="n"/>
+      <c r="E572" s="60" t="n"/>
+      <c r="F572" s="60" t="n"/>
+      <c r="G572" s="60" t="n"/>
+      <c r="H572" s="60" t="n"/>
+      <c r="I572" s="60" t="n"/>
+      <c r="J572" s="60" t="n"/>
+      <c r="K572" s="60" t="n"/>
+      <c r="L572" s="61">
+        <f>SUM(L5:L571)</f>
+        <v/>
+      </c>
+      <c r="M572" s="60" t="n"/>
+      <c r="N572" s="60" t="n"/>
+      <c r="O572" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P569" s="60" t="n"/>
-      <c r="Q569" s="60" t="n"/>
+      <c r="P572" s="60" t="n"/>
+      <c r="Q572" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -38999,17 +39179,47 @@
       <c r="M59" s="47" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="99">
-      <c r="A60" s="43" t="n"/>
-      <c r="B60" s="53" t="n"/>
-      <c r="C60" s="55" t="n"/>
-      <c r="D60" s="55" t="n"/>
-      <c r="E60" s="55" t="n"/>
-      <c r="F60" s="55" t="n"/>
-      <c r="G60" s="63" t="n"/>
-      <c r="H60" s="55" t="n"/>
+      <c r="A60" s="43" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="53" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C60" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D60" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E60" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F60" s="55" t="inlineStr">
+        <is>
+          <t>Ultratech Super+Plain cement, transport</t>
+        </is>
+      </c>
+      <c r="G60" s="63" t="n">
+        <v>12210</v>
+      </c>
+      <c r="H60" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I60" s="55" t="n"/>
       <c r="J60" s="55" t="n"/>
-      <c r="K60" s="55" t="n"/>
+      <c r="K60" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L60" s="58" t="n"/>
       <c r="M60" s="55" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add: ₹1,00,000 advance to Econ Builder (Avinash, 12-Sep)
Generalize reconciliation gap check to support advance credit on any
vendor, not just Brick Company — previously hardcoded to brickAdvance.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -39224,17 +39224,47 @@
       <c r="M60" s="55" t="n"/>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="99">
-      <c r="A61" s="41" t="n"/>
-      <c r="B61" s="45" t="n"/>
-      <c r="C61" s="47" t="n"/>
-      <c r="D61" s="47" t="n"/>
-      <c r="E61" s="47" t="n"/>
-      <c r="F61" s="47" t="n"/>
-      <c r="G61" s="62" t="n"/>
-      <c r="H61" s="47" t="n"/>
+      <c r="A61" s="41" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="45" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C61" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D61" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E61" s="47" t="inlineStr">
+        <is>
+          <t>Advance</t>
+        </is>
+      </c>
+      <c r="F61" s="47" t="inlineStr">
+        <is>
+          <t>Advance for upcoming work — to be adjusted against future bills</t>
+        </is>
+      </c>
+      <c r="G61" s="62" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H61" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I61" s="47" t="n"/>
       <c r="J61" s="47" t="n"/>
-      <c r="K61" s="47" t="n"/>
+      <c r="K61" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L61" s="50" t="n"/>
       <c r="M61" s="47" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix: ₹1,00,000 Econ Builder payment was for work done, not an advance
Added matching ₹1,00,000 transaction (Professional Fees / Engineer
Supervision — general site work, 12-Sep) so the payment settles
against actual billed work instead of sitting as unmatched advance.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -1466,7 +1466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -2466,7 +2466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="99" min="1" max="1"/>
     <col width="12" customWidth="1" style="99" min="2" max="2"/>
@@ -2946,7 +2946,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="8" customWidth="1" style="99" min="2" max="2"/>
@@ -3032,7 +3032,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="2" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>
@@ -5053,7 +5053,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -6539,8 +6539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R572"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <dimension ref="A1:R573"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -24613,33 +24613,93 @@
       </c>
     </row>
     <row r="572">
-      <c r="A572" s="60" t="inlineStr">
+      <c r="A572" t="n">
+        <v>566</v>
+      </c>
+      <c r="B572" s="128" t="n">
+        <v>46277</v>
+      </c>
+      <c r="C572">
+        <f>IF(B572="","",TEXT(B572,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>Construction work done — general site supervision &amp; labour (Sep)</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I572" t="n">
+        <v>1</v>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K572" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L572">
+        <f>I572*K572</f>
+        <v/>
+      </c>
+      <c r="N572">
+        <f>M572*L572</f>
+        <v/>
+      </c>
+      <c r="O572">
+        <f>IF(L572="","",IF(M572="",L572,L572*(1-M572)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B572" s="60" t="n"/>
-      <c r="C572" s="60" t="n"/>
-      <c r="D572" s="60" t="n"/>
-      <c r="E572" s="60" t="n"/>
-      <c r="F572" s="60" t="n"/>
-      <c r="G572" s="60" t="n"/>
-      <c r="H572" s="60" t="n"/>
-      <c r="I572" s="60" t="n"/>
-      <c r="J572" s="60" t="n"/>
-      <c r="K572" s="60" t="n"/>
-      <c r="L572" s="61">
-        <f>SUM(L5:L571)</f>
-        <v/>
-      </c>
-      <c r="M572" s="60" t="n"/>
-      <c r="N572" s="60" t="n"/>
-      <c r="O572" s="61">
+      <c r="B573" s="60" t="n"/>
+      <c r="C573" s="60" t="n"/>
+      <c r="D573" s="60" t="n"/>
+      <c r="E573" s="60" t="n"/>
+      <c r="F573" s="60" t="n"/>
+      <c r="G573" s="60" t="n"/>
+      <c r="H573" s="60" t="n"/>
+      <c r="I573" s="60" t="n"/>
+      <c r="J573" s="60" t="n"/>
+      <c r="K573" s="60" t="n"/>
+      <c r="L573" s="61">
+        <f>SUM(L5:L572)</f>
+        <v/>
+      </c>
+      <c r="M573" s="60" t="n"/>
+      <c r="N573" s="60" t="n"/>
+      <c r="O573" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P572" s="60" t="n"/>
-      <c r="Q572" s="60" t="n"/>
+      <c r="P573" s="60" t="n"/>
+      <c r="Q573" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -24682,7 +24742,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -36589,7 +36649,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M505"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -39242,12 +39302,12 @@
       </c>
       <c r="E61" s="47" t="inlineStr">
         <is>
-          <t>Advance</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F61" s="47" t="inlineStr">
         <is>
-          <t>Advance for upcoming work — to be adjusted against future bills</t>
+          <t>Construction work done — general site supervision &amp; labour (Sep)</t>
         </is>
       </c>
       <c r="G61" s="62" t="n">
@@ -47987,7 +48047,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -49331,7 +49391,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="3"/>
@@ -58005,7 +58065,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>

</xml_diff>

<commit_message>
Add: ₹57,200 Sand Truck Wala (Avinash, 22-Sep) — 944 CFT @ ₹60.59/CFT
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -1466,7 +1466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -2466,7 +2466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="99" min="1" max="1"/>
     <col width="12" customWidth="1" style="99" min="2" max="2"/>
@@ -2946,7 +2946,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="8" customWidth="1" style="99" min="2" max="2"/>
@@ -3032,7 +3032,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="2" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>
@@ -5053,7 +5053,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -6539,8 +6539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R606"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <dimension ref="A1:R607"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -30487,33 +30487,93 @@
       </c>
     </row>
     <row r="606">
-      <c r="A606" s="60" t="inlineStr">
+      <c r="A606" t="n">
+        <v>614</v>
+      </c>
+      <c r="B606" s="128" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C606">
+        <f>IF(B606="","",TEXT(B606,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>Sand Truck — 944 CFT @ ₹60.59/CFT</t>
+        </is>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="I606" t="n">
+        <v>944</v>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>CFT</t>
+        </is>
+      </c>
+      <c r="K606" t="n">
+        <v>60.59322033898305</v>
+      </c>
+      <c r="L606">
+        <f>IF(OR(I606="",K606=""),"",I606*K606)</f>
+        <v/>
+      </c>
+      <c r="N606">
+        <f>M606*L606</f>
+        <v/>
+      </c>
+      <c r="O606">
+        <f>IF(L606="","",IF(M606="",L606,L606*(1-M606)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B606" s="60" t="n"/>
-      <c r="C606" s="60" t="n"/>
-      <c r="D606" s="60" t="n"/>
-      <c r="E606" s="60" t="n"/>
-      <c r="F606" s="60" t="n"/>
-      <c r="G606" s="60" t="n"/>
-      <c r="H606" s="60" t="n"/>
-      <c r="I606" s="60" t="n"/>
-      <c r="J606" s="60" t="n"/>
-      <c r="K606" s="60" t="n"/>
-      <c r="L606" s="61">
-        <f>SUM(L5:L605)</f>
-        <v/>
-      </c>
-      <c r="M606" s="60" t="n"/>
-      <c r="N606" s="60" t="n"/>
-      <c r="O606" s="61">
+      <c r="B607" s="60" t="n"/>
+      <c r="C607" s="60" t="n"/>
+      <c r="D607" s="60" t="n"/>
+      <c r="E607" s="60" t="n"/>
+      <c r="F607" s="60" t="n"/>
+      <c r="G607" s="60" t="n"/>
+      <c r="H607" s="60" t="n"/>
+      <c r="I607" s="60" t="n"/>
+      <c r="J607" s="60" t="n"/>
+      <c r="K607" s="60" t="n"/>
+      <c r="L607" s="61">
+        <f>SUM(L5:L606)</f>
+        <v/>
+      </c>
+      <c r="M607" s="60" t="n"/>
+      <c r="N607" s="60" t="n"/>
+      <c r="O607" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P606" s="60" t="n"/>
-      <c r="Q606" s="60" t="n"/>
+      <c r="P607" s="60" t="n"/>
+      <c r="Q607" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -30556,7 +30616,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -42463,7 +42523,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M495"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -46832,16 +46892,44 @@
       <c r="A99" s="41" t="n">
         <v>105</v>
       </c>
-      <c r="B99" s="45" t="n"/>
-      <c r="C99" s="47" t="n"/>
-      <c r="D99" s="47" t="n"/>
-      <c r="E99" s="47" t="n"/>
-      <c r="F99" s="47" t="n"/>
-      <c r="G99" s="62" t="n"/>
-      <c r="H99" s="47" t="n"/>
+      <c r="B99" s="45" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C99" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D99" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="E99" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F99" s="47" t="inlineStr">
+        <is>
+          <t>Sand Truck — 944 CFT</t>
+        </is>
+      </c>
+      <c r="G99" s="62" t="n">
+        <v>57200</v>
+      </c>
+      <c r="H99" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I99" s="47" t="n"/>
       <c r="J99" s="47" t="n"/>
-      <c r="K99" s="47" t="n"/>
+      <c r="K99" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L99" s="50">
         <f>IF(G109="","",IF(L108="",G109,L108+G109))</f>
         <v/>
@@ -54806,7 +54894,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -56150,7 +56238,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="3"/>
@@ -64824,7 +64912,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>

</xml_diff>

<commit_message>
Add: ₹50,000 Econ Builder (Papa, 28-Sep) and ₹79,500 gitti (Avinash, 1-Oct)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -1466,7 +1466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D110"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -2466,7 +2466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="99" min="1" max="1"/>
     <col width="12" customWidth="1" style="99" min="2" max="2"/>
@@ -2946,7 +2946,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="8" customWidth="1" style="99" min="2" max="2"/>
@@ -3032,7 +3032,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>
@@ -5053,7 +5053,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -6539,8 +6539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R607"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:R609"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -30547,33 +30547,153 @@
       </c>
     </row>
     <row r="607">
-      <c r="A607" s="60" t="inlineStr">
+      <c r="A607" t="n">
+        <v>615</v>
+      </c>
+      <c r="B607" s="128" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C607">
+        <f>IF(B607="","",TEXT(B607,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>Construction work done — general site supervision &amp; labour (Papa, 28-Sep)</t>
+        </is>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I607" t="n">
+        <v>1</v>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K607" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L607">
+        <f>IF(OR(I607="",K607=""),"",I607*K607)</f>
+        <v/>
+      </c>
+      <c r="N607">
+        <f>M607*L607</f>
+        <v/>
+      </c>
+      <c r="O607">
+        <f>IF(L607="","",IF(M607="",L607,L607*(1-M607)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="n">
+        <v>616</v>
+      </c>
+      <c r="B608" s="128" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C608">
+        <f>IF(B608="","",TEXT(B608,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Concrete/Gitti</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>Gitti delivery (qty not recorded)</t>
+        </is>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="I608" t="n">
+        <v>1</v>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K608" t="n">
+        <v>79500</v>
+      </c>
+      <c r="L608">
+        <f>IF(OR(I608="",K608=""),"",I608*K608)</f>
+        <v/>
+      </c>
+      <c r="N608">
+        <f>M608*L608</f>
+        <v/>
+      </c>
+      <c r="O608">
+        <f>IF(L608="","",IF(M608="",L608,L608*(1-M608)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B607" s="60" t="n"/>
-      <c r="C607" s="60" t="n"/>
-      <c r="D607" s="60" t="n"/>
-      <c r="E607" s="60" t="n"/>
-      <c r="F607" s="60" t="n"/>
-      <c r="G607" s="60" t="n"/>
-      <c r="H607" s="60" t="n"/>
-      <c r="I607" s="60" t="n"/>
-      <c r="J607" s="60" t="n"/>
-      <c r="K607" s="60" t="n"/>
-      <c r="L607" s="61">
-        <f>SUM(L5:L606)</f>
-        <v/>
-      </c>
-      <c r="M607" s="60" t="n"/>
-      <c r="N607" s="60" t="n"/>
-      <c r="O607" s="61">
+      <c r="B609" s="60" t="n"/>
+      <c r="C609" s="60" t="n"/>
+      <c r="D609" s="60" t="n"/>
+      <c r="E609" s="60" t="n"/>
+      <c r="F609" s="60" t="n"/>
+      <c r="G609" s="60" t="n"/>
+      <c r="H609" s="60" t="n"/>
+      <c r="I609" s="60" t="n"/>
+      <c r="J609" s="60" t="n"/>
+      <c r="K609" s="60" t="n"/>
+      <c r="L609" s="61">
+        <f>SUM(L5:L608)</f>
+        <v/>
+      </c>
+      <c r="M609" s="60" t="n"/>
+      <c r="N609" s="60" t="n"/>
+      <c r="O609" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P607" s="60" t="n"/>
-      <c r="Q607" s="60" t="n"/>
+      <c r="P609" s="60" t="n"/>
+      <c r="Q609" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -30616,7 +30736,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -42523,7 +42643,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M495"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="2"/>
@@ -46940,16 +47060,44 @@
       <c r="A100" s="43" t="n">
         <v>106</v>
       </c>
-      <c r="B100" s="53" t="n"/>
-      <c r="C100" s="55" t="n"/>
-      <c r="D100" s="55" t="n"/>
-      <c r="E100" s="55" t="n"/>
-      <c r="F100" s="55" t="n"/>
-      <c r="G100" s="63" t="n"/>
-      <c r="H100" s="55" t="n"/>
+      <c r="B100" s="53" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C100" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D100" s="55" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E100" s="55" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F100" s="55" t="inlineStr">
+        <is>
+          <t>Construction work done — general (Papa, 28-Sep)</t>
+        </is>
+      </c>
+      <c r="G100" s="63" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H100" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I100" s="55" t="n"/>
       <c r="J100" s="55" t="n"/>
-      <c r="K100" s="55" t="n"/>
+      <c r="K100" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L100" s="58">
         <f>IF(G110="","",IF(L109="",G110,L109+G110))</f>
         <v/>
@@ -46960,16 +47108,44 @@
       <c r="A101" s="41" t="n">
         <v>107</v>
       </c>
-      <c r="B101" s="45" t="n"/>
-      <c r="C101" s="47" t="n"/>
-      <c r="D101" s="47" t="n"/>
-      <c r="E101" s="47" t="n"/>
-      <c r="F101" s="47" t="n"/>
-      <c r="G101" s="62" t="n"/>
-      <c r="H101" s="47" t="n"/>
+      <c r="B101" s="45" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C101" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D101" s="47" t="inlineStr">
+        <is>
+          <t>Concrete Supplier</t>
+        </is>
+      </c>
+      <c r="E101" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F101" s="47" t="inlineStr">
+        <is>
+          <t>Gitti delivery</t>
+        </is>
+      </c>
+      <c r="G101" s="62" t="n">
+        <v>79500</v>
+      </c>
+      <c r="H101" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I101" s="47" t="n"/>
       <c r="J101" s="47" t="n"/>
-      <c r="K101" s="47" t="n"/>
+      <c r="K101" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L101" s="50">
         <f>IF(G111="","",IF(L110="",G111,L110+G111))</f>
         <v/>
@@ -54894,7 +55070,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
     <col width="28" customWidth="1" style="99" min="2" max="2"/>
@@ -56238,7 +56414,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
     <col width="14" customWidth="1" style="99" min="2" max="3"/>
@@ -64912,7 +65088,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
     <col width="18" customWidth="1" style="99" min="2" max="2"/>

</xml_diff>

<commit_message>
Add: Pappu Hardware 5-Oct bill ₹4,66,024 (steel, cement, misc); ₹4.5L paid by Avinash, ₹16,024 due
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R609"/>
+  <dimension ref="A1:R630"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -30667,33 +30667,1293 @@
       </c>
     </row>
     <row r="609">
-      <c r="A609" s="60" t="inlineStr">
+      <c r="A609" t="n">
+        <v>617</v>
+      </c>
+      <c r="B609" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C609">
+        <f>IF(B609="","",TEXT(B609,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Tiscon 16mm</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>Tiscon 16mm rod 6 pcs</t>
+        </is>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I609" t="n">
+        <v>6</v>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K609" t="n">
+        <v>1459.166666666667</v>
+      </c>
+      <c r="L609">
+        <f>IF(OR(I609="",K609=""),"",I609*K609)</f>
+        <v/>
+      </c>
+      <c r="N609">
+        <f>M609*L609</f>
+        <v/>
+      </c>
+      <c r="O609">
+        <f>IF(L609="","",IF(M609="",L609,L609*(1-M609)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="n">
+        <v>618</v>
+      </c>
+      <c r="B610" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C610">
+        <f>IF(B610="","",TEXT(B610,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm rod 50 pcs</t>
+        </is>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I610" t="n">
+        <v>50</v>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K610" t="n">
+        <v>819.84</v>
+      </c>
+      <c r="L610">
+        <f>IF(OR(I610="",K610=""),"",I610*K610)</f>
+        <v/>
+      </c>
+      <c r="N610">
+        <f>M610*L610</f>
+        <v/>
+      </c>
+      <c r="O610">
+        <f>IF(L610="","",IF(M610="",L610,L610*(1-M610)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="n">
+        <v>619</v>
+      </c>
+      <c r="B611" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C611">
+        <f>IF(B611="","",TEXT(B611,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm</t>
+        </is>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm rod 260 pcs</t>
+        </is>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I611" t="n">
+        <v>260</v>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K611" t="n">
+        <v>580.8</v>
+      </c>
+      <c r="L611">
+        <f>IF(OR(I611="",K611=""),"",I611*K611)</f>
+        <v/>
+      </c>
+      <c r="N611">
+        <f>M611*L611</f>
+        <v/>
+      </c>
+      <c r="O611">
+        <f>IF(L611="","",IF(M611="",L611,L611*(1-M611)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="n">
+        <v>620</v>
+      </c>
+      <c r="B612" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C612">
+        <f>IF(B612="","",TEXT(B612,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm</t>
+        </is>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm rod 202 pcs</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I612" t="n">
+        <v>202</v>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K612" t="n">
+        <v>380.1584158415841</v>
+      </c>
+      <c r="L612">
+        <f>IF(OR(I612="",K612=""),"",I612*K612)</f>
+        <v/>
+      </c>
+      <c r="N612">
+        <f>M612*L612</f>
+        <v/>
+      </c>
+      <c r="O612">
+        <f>IF(L612="","",IF(M612="",L612,L612*(1-M612)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="n">
+        <v>621</v>
+      </c>
+      <c r="B613" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C613">
+        <f>IF(B613="","",TEXT(B613,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm rod 50 pcs</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I613" t="n">
+        <v>50</v>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K613" t="n">
+        <v>233</v>
+      </c>
+      <c r="L613">
+        <f>IF(OR(I613="",K613=""),"",I613*K613)</f>
+        <v/>
+      </c>
+      <c r="N613">
+        <f>M613*L613</f>
+        <v/>
+      </c>
+      <c r="O613">
+        <f>IF(L613="","",IF(M613="",L613,L613*(1-M613)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="n">
+        <v>622</v>
+      </c>
+      <c r="B614" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C614">
+        <f>IF(B614="","",TEXT(B614,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Binding Wire</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>Binding wire</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I614" t="n">
+        <v>1</v>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K614" t="n">
+        <v>1700</v>
+      </c>
+      <c r="L614">
+        <f>IF(OR(I614="",K614=""),"",I614*K614)</f>
+        <v/>
+      </c>
+      <c r="N614">
+        <f>M614*L614</f>
+        <v/>
+      </c>
+      <c r="O614">
+        <f>IF(L614="","",IF(M614="",L614,L614*(1-M614)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="n">
+        <v>623</v>
+      </c>
+      <c r="B615" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C615">
+        <f>IF(B615="","",TEXT(B615,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I615" t="n">
+        <v>1</v>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K615" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L615">
+        <f>IF(OR(I615="",K615=""),"",I615*K615)</f>
+        <v/>
+      </c>
+      <c r="N615">
+        <f>M615*L615</f>
+        <v/>
+      </c>
+      <c r="O615">
+        <f>IF(L615="","",IF(M615="",L615,L615*(1-M615)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="n">
+        <v>624</v>
+      </c>
+      <c r="B616" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C616">
+        <f>IF(B616="","",TEXT(B616,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I616" t="n">
+        <v>1</v>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K616" t="n">
+        <v>900</v>
+      </c>
+      <c r="L616">
+        <f>IF(OR(I616="",K616=""),"",I616*K616)</f>
+        <v/>
+      </c>
+      <c r="N616">
+        <f>M616*L616</f>
+        <v/>
+      </c>
+      <c r="O616">
+        <f>IF(L616="","",IF(M616="",L616,L616*(1-M616)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="n">
+        <v>625</v>
+      </c>
+      <c r="B617" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C617">
+        <f>IF(B617="","",TEXT(B617,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm rod 60 pcs</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I617" t="n">
+        <v>60</v>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K617" t="n">
+        <v>391.6833333333333</v>
+      </c>
+      <c r="L617">
+        <f>IF(OR(I617="",K617=""),"",I617*K617)</f>
+        <v/>
+      </c>
+      <c r="N617">
+        <f>M617*L617</f>
+        <v/>
+      </c>
+      <c r="O617">
+        <f>IF(L617="","",IF(M617="",L617,L617*(1-M617)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="n">
+        <v>626</v>
+      </c>
+      <c r="B618" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C618">
+        <f>IF(B618="","",TEXT(B618,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I618" t="n">
+        <v>1</v>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K618" t="n">
+        <v>350</v>
+      </c>
+      <c r="L618">
+        <f>IF(OR(I618="",K618=""),"",I618*K618)</f>
+        <v/>
+      </c>
+      <c r="N618">
+        <f>M618*L618</f>
+        <v/>
+      </c>
+      <c r="O618">
+        <f>IF(L618="","",IF(M618="",L618,L618*(1-M618)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="n">
+        <v>627</v>
+      </c>
+      <c r="B619" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C619">
+        <f>IF(B619="","",TEXT(B619,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm rod 24 pcs</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I619" t="n">
+        <v>24</v>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K619" t="n">
+        <v>240</v>
+      </c>
+      <c r="L619">
+        <f>IF(OR(I619="",K619=""),"",I619*K619)</f>
+        <v/>
+      </c>
+      <c r="N619">
+        <f>M619*L619</f>
+        <v/>
+      </c>
+      <c r="O619">
+        <f>IF(L619="","",IF(M619="",L619,L619*(1-M619)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="n">
+        <v>628</v>
+      </c>
+      <c r="B620" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C620">
+        <f>IF(B620="","",TEXT(B620,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I620" t="n">
+        <v>1</v>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K620" t="n">
+        <v>340</v>
+      </c>
+      <c r="L620">
+        <f>IF(OR(I620="",K620=""),"",I620*K620)</f>
+        <v/>
+      </c>
+      <c r="N620">
+        <f>M620*L620</f>
+        <v/>
+      </c>
+      <c r="O620">
+        <f>IF(L620="","",IF(M620="",L620,L620*(1-M620)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="n">
+        <v>629</v>
+      </c>
+      <c r="B621" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C621">
+        <f>IF(B621="","",TEXT(B621,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>Tiscon 6mm rod 48 pcs</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I621" t="n">
+        <v>48</v>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K621" t="n">
+        <v>240</v>
+      </c>
+      <c r="L621">
+        <f>IF(OR(I621="",K621=""),"",I621*K621)</f>
+        <v/>
+      </c>
+      <c r="N621">
+        <f>M621*L621</f>
+        <v/>
+      </c>
+      <c r="O621">
+        <f>IF(L621="","",IF(M621="",L621,L621*(1-M621)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="n">
+        <v>630</v>
+      </c>
+      <c r="B622" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C622">
+        <f>IF(B622="","",TEXT(B622,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm rod 6 pcs</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I622" t="n">
+        <v>6</v>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K622" t="n">
+        <v>866</v>
+      </c>
+      <c r="L622">
+        <f>IF(OR(I622="",K622=""),"",I622*K622)</f>
+        <v/>
+      </c>
+      <c r="N622">
+        <f>M622*L622</f>
+        <v/>
+      </c>
+      <c r="O622">
+        <f>IF(L622="","",IF(M622="",L622,L622*(1-M622)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="n">
+        <v>631</v>
+      </c>
+      <c r="B623" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C623">
+        <f>IF(B623="","",TEXT(B623,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I623" t="n">
+        <v>1</v>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K623" t="n">
+        <v>350</v>
+      </c>
+      <c r="L623">
+        <f>IF(OR(I623="",K623=""),"",I623*K623)</f>
+        <v/>
+      </c>
+      <c r="N623">
+        <f>M623*L623</f>
+        <v/>
+      </c>
+      <c r="O623">
+        <f>IF(L623="","",IF(M623="",L623,L623*(1-M623)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="n">
+        <v>632</v>
+      </c>
+      <c r="B624" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C624">
+        <f>IF(B624="","",TEXT(B624,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Misc Expense</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I624" t="n">
+        <v>1</v>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K624" t="n">
+        <v>1170</v>
+      </c>
+      <c r="L624">
+        <f>IF(OR(I624="",K624=""),"",I624*K624)</f>
+        <v/>
+      </c>
+      <c r="N624">
+        <f>M624*L624</f>
+        <v/>
+      </c>
+      <c r="O624">
+        <f>IF(L624="","",IF(M624="",L624,L624*(1-M624)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="n">
+        <v>633</v>
+      </c>
+      <c r="B625" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C625">
+        <f>IF(B625="","",TEXT(B625,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Rings</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>Rings (stirrups)</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I625" t="n">
+        <v>1</v>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K625" t="n">
+        <v>4040</v>
+      </c>
+      <c r="L625">
+        <f>IF(OR(I625="",K625=""),"",I625*K625)</f>
+        <v/>
+      </c>
+      <c r="N625">
+        <f>M625*L625</f>
+        <v/>
+      </c>
+      <c r="O625">
+        <f>IF(L625="","",IF(M625="",L625,L625*(1-M625)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="n">
+        <v>634</v>
+      </c>
+      <c r="B626" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C626">
+        <f>IF(B626="","",TEXT(B626,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>Ultratech Weatherplus cement 300 bags @ ₹370</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I626" t="n">
+        <v>300</v>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K626" t="n">
+        <v>370</v>
+      </c>
+      <c r="L626">
+        <f>IF(OR(I626="",K626=""),"",I626*K626)</f>
+        <v/>
+      </c>
+      <c r="N626">
+        <f>M626*L626</f>
+        <v/>
+      </c>
+      <c r="O626">
+        <f>IF(L626="","",IF(M626="",L626,L626*(1-M626)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="n">
+        <v>635</v>
+      </c>
+      <c r="B627" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C627">
+        <f>IF(B627="","",TEXT(B627,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I627" t="n">
+        <v>1</v>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K627" t="n">
+        <v>900</v>
+      </c>
+      <c r="L627">
+        <f>IF(OR(I627="",K627=""),"",I627*K627)</f>
+        <v/>
+      </c>
+      <c r="N627">
+        <f>M627*L627</f>
+        <v/>
+      </c>
+      <c r="O627">
+        <f>IF(L627="","",IF(M627="",L627,L627*(1-M627)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="n">
+        <v>636</v>
+      </c>
+      <c r="B628" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C628">
+        <f>IF(B628="","",TEXT(B628,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Misc Expense</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I628" t="n">
+        <v>1</v>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K628" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L628">
+        <f>IF(OR(I628="",K628=""),"",I628*K628)</f>
+        <v/>
+      </c>
+      <c r="N628">
+        <f>M628*L628</f>
+        <v/>
+      </c>
+      <c r="O628">
+        <f>IF(L628="","",IF(M628="",L628,L628*(1-M628)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="n">
+        <v>637</v>
+      </c>
+      <c r="B629" s="128" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C629">
+        <f>IF(B629="","",TEXT(B629,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Dr Fixit</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>Dr Fixit 40 litres</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I629" t="n">
+        <v>40</v>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>Litres</t>
+        </is>
+      </c>
+      <c r="K629" t="n">
+        <v>140</v>
+      </c>
+      <c r="L629">
+        <f>IF(OR(I629="",K629=""),"",I629*K629)</f>
+        <v/>
+      </c>
+      <c r="N629">
+        <f>M629*L629</f>
+        <v/>
+      </c>
+      <c r="O629">
+        <f>IF(L629="","",IF(M629="",L629,L629*(1-M629)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B609" s="60" t="n"/>
-      <c r="C609" s="60" t="n"/>
-      <c r="D609" s="60" t="n"/>
-      <c r="E609" s="60" t="n"/>
-      <c r="F609" s="60" t="n"/>
-      <c r="G609" s="60" t="n"/>
-      <c r="H609" s="60" t="n"/>
-      <c r="I609" s="60" t="n"/>
-      <c r="J609" s="60" t="n"/>
-      <c r="K609" s="60" t="n"/>
-      <c r="L609" s="61">
-        <f>SUM(L5:L608)</f>
-        <v/>
-      </c>
-      <c r="M609" s="60" t="n"/>
-      <c r="N609" s="60" t="n"/>
-      <c r="O609" s="61">
+      <c r="B630" s="60" t="n"/>
+      <c r="C630" s="60" t="n"/>
+      <c r="D630" s="60" t="n"/>
+      <c r="E630" s="60" t="n"/>
+      <c r="F630" s="60" t="n"/>
+      <c r="G630" s="60" t="n"/>
+      <c r="H630" s="60" t="n"/>
+      <c r="I630" s="60" t="n"/>
+      <c r="J630" s="60" t="n"/>
+      <c r="K630" s="60" t="n"/>
+      <c r="L630" s="61">
+        <f>SUM(L5:L629)</f>
+        <v/>
+      </c>
+      <c r="M630" s="60" t="n"/>
+      <c r="N630" s="60" t="n"/>
+      <c r="O630" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P609" s="60" t="n"/>
-      <c r="Q609" s="60" t="n"/>
+      <c r="P630" s="60" t="n"/>
+      <c r="Q630" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -47156,16 +48416,44 @@
       <c r="A102" s="43" t="n">
         <v>108</v>
       </c>
-      <c r="B102" s="53" t="n"/>
-      <c r="C102" s="55" t="n"/>
-      <c r="D102" s="55" t="n"/>
-      <c r="E102" s="55" t="n"/>
-      <c r="F102" s="55" t="n"/>
-      <c r="G102" s="63" t="n"/>
-      <c r="H102" s="55" t="n"/>
+      <c r="B102" s="53" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C102" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D102" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E102" s="55" t="inlineStr">
+        <is>
+          <t>Steel / Iron + Cement + Building Materials</t>
+        </is>
+      </c>
+      <c r="F102" s="55" t="inlineStr">
+        <is>
+          <t>Part payment against 5-Oct bill (₹4,66,024)</t>
+        </is>
+      </c>
+      <c r="G102" s="63" t="n">
+        <v>450000</v>
+      </c>
+      <c r="H102" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I102" s="55" t="n"/>
       <c r="J102" s="55" t="n"/>
-      <c r="K102" s="55" t="n"/>
+      <c r="K102" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L102" s="58">
         <f>IF(G112="","",IF(L111="",G112,L111+G112))</f>
         <v/>

</xml_diff>

<commit_message>
Add: Pappu Hardware 6-Oct delivery ₹61,329 (12mm/10mm rods, labour), payment pending
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R630"/>
+  <dimension ref="A1:R633"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -31927,33 +31927,213 @@
       </c>
     </row>
     <row r="630">
-      <c r="A630" s="60" t="inlineStr">
+      <c r="A630" t="n">
+        <v>638</v>
+      </c>
+      <c r="B630" s="128" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C630">
+        <f>IF(B630="","",TEXT(B630,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm rod 2 pcs @ ₹902 (4% disc → ₹865.92)</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I630" t="n">
+        <v>2</v>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K630" t="n">
+        <v>865.92</v>
+      </c>
+      <c r="L630">
+        <f>IF(OR(I630="",K630=""),"",I630*K630)</f>
+        <v/>
+      </c>
+      <c r="N630">
+        <f>M630*L630</f>
+        <v/>
+      </c>
+      <c r="O630">
+        <f>IF(L630="","",IF(M630="",L630,L630*(1-M630)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="n">
+        <v>639</v>
+      </c>
+      <c r="B631" s="128" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C631">
+        <f>IF(B631="","",TEXT(B631,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm rod 96 pcs @ ₹642 (4% disc → ₹616.32)</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I631" t="n">
+        <v>96</v>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K631" t="n">
+        <v>616.3200000000001</v>
+      </c>
+      <c r="L631">
+        <f>IF(OR(I631="",K631=""),"",I631*K631)</f>
+        <v/>
+      </c>
+      <c r="N631">
+        <f>M631*L631</f>
+        <v/>
+      </c>
+      <c r="O631">
+        <f>IF(L631="","",IF(M631="",L631,L631*(1-M631)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="n">
+        <v>640</v>
+      </c>
+      <c r="B632" s="128" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C632">
+        <f>IF(B632="","",TEXT(B632,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I632" t="n">
+        <v>1</v>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K632" t="n">
+        <v>430</v>
+      </c>
+      <c r="L632">
+        <f>IF(OR(I632="",K632=""),"",I632*K632)</f>
+        <v/>
+      </c>
+      <c r="N632">
+        <f>M632*L632</f>
+        <v/>
+      </c>
+      <c r="O632">
+        <f>IF(L632="","",IF(M632="",L632,L632*(1-M632)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B630" s="60" t="n"/>
-      <c r="C630" s="60" t="n"/>
-      <c r="D630" s="60" t="n"/>
-      <c r="E630" s="60" t="n"/>
-      <c r="F630" s="60" t="n"/>
-      <c r="G630" s="60" t="n"/>
-      <c r="H630" s="60" t="n"/>
-      <c r="I630" s="60" t="n"/>
-      <c r="J630" s="60" t="n"/>
-      <c r="K630" s="60" t="n"/>
-      <c r="L630" s="61">
-        <f>SUM(L5:L629)</f>
-        <v/>
-      </c>
-      <c r="M630" s="60" t="n"/>
-      <c r="N630" s="60" t="n"/>
-      <c r="O630" s="61">
+      <c r="B633" s="60" t="n"/>
+      <c r="C633" s="60" t="n"/>
+      <c r="D633" s="60" t="n"/>
+      <c r="E633" s="60" t="n"/>
+      <c r="F633" s="60" t="n"/>
+      <c r="G633" s="60" t="n"/>
+      <c r="H633" s="60" t="n"/>
+      <c r="I633" s="60" t="n"/>
+      <c r="J633" s="60" t="n"/>
+      <c r="K633" s="60" t="n"/>
+      <c r="L633" s="61">
+        <f>SUM(L5:L632)</f>
+        <v/>
+      </c>
+      <c r="M633" s="60" t="n"/>
+      <c r="N633" s="60" t="n"/>
+      <c r="O633" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P630" s="60" t="n"/>
-      <c r="Q630" s="60" t="n"/>
+      <c r="P633" s="60" t="n"/>
+      <c r="Q633" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>

</xml_diff>

<commit_message>
Add: gate-frame wood ₹69,378 (Khutauna Chirai mill, 7-Oct) tagged C/B unit; C-unit costs now exceed B
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R633"/>
+  <dimension ref="A1:R643"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -32107,33 +32107,683 @@
       </c>
     </row>
     <row r="633">
-      <c r="A633" s="60" t="inlineStr">
+      <c r="A633" t="n">
+        <v>641</v>
+      </c>
+      <c r="B633" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C633">
+        <f>IF(B633="","",TEXT(B633,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>5 inch 7 feet wood × 6 pcs (gate frame, C unit)</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I633" t="n">
+        <v>4.375</v>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K633" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L633">
+        <f>IF(OR(I633="",K633=""),"",I633*K633)</f>
+        <v/>
+      </c>
+      <c r="N633">
+        <f>M633*L633</f>
+        <v/>
+      </c>
+      <c r="O633">
+        <f>IF(L633="","",IF(M633="",L633,L633*(1-M633)))</f>
+        <v/>
+      </c>
+      <c r="R633" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="n">
+        <v>642</v>
+      </c>
+      <c r="B634" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C634">
+        <f>IF(B634="","",TEXT(B634,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>4 inch 7 feet wood × 10 pcs (gate frame, C unit)</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I634" t="n">
+        <v>5.833333333333333</v>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K634" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L634">
+        <f>IF(OR(I634="",K634=""),"",I634*K634)</f>
+        <v/>
+      </c>
+      <c r="N634">
+        <f>M634*L634</f>
+        <v/>
+      </c>
+      <c r="O634">
+        <f>IF(L634="","",IF(M634="",L634,L634*(1-M634)))</f>
+        <v/>
+      </c>
+      <c r="R634" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="n">
+        <v>643</v>
+      </c>
+      <c r="B635" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C635">
+        <f>IF(B635="","",TEXT(B635,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>5 inch 3.5 feet wood × 3 pcs (gate frame, C unit)</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I635" t="n">
+        <v>1.09375</v>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K635" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L635">
+        <f>IF(OR(I635="",K635=""),"",I635*K635)</f>
+        <v/>
+      </c>
+      <c r="N635">
+        <f>M635*L635</f>
+        <v/>
+      </c>
+      <c r="O635">
+        <f>IF(L635="","",IF(M635="",L635,L635*(1-M635)))</f>
+        <v/>
+      </c>
+      <c r="R635" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="n">
+        <v>644</v>
+      </c>
+      <c r="B636" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C636">
+        <f>IF(B636="","",TEXT(B636,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>4 inch 3.5 feet wood × 5 pcs (gate frame, C unit)</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I636" t="n">
+        <v>1.458333333333333</v>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K636" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L636">
+        <f>IF(OR(I636="",K636=""),"",I636*K636)</f>
+        <v/>
+      </c>
+      <c r="N636">
+        <f>M636*L636</f>
+        <v/>
+      </c>
+      <c r="O636">
+        <f>IF(L636="","",IF(M636="",L636,L636*(1-M636)))</f>
+        <v/>
+      </c>
+      <c r="R636" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="n">
+        <v>645</v>
+      </c>
+      <c r="B637" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C637">
+        <f>IF(B637="","",TEXT(B637,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>Labour (gate frame wood, C unit)</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I637" t="n">
+        <v>1</v>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K637" t="n">
+        <v>400</v>
+      </c>
+      <c r="L637">
+        <f>IF(OR(I637="",K637=""),"",I637*K637)</f>
+        <v/>
+      </c>
+      <c r="N637">
+        <f>M637*L637</f>
+        <v/>
+      </c>
+      <c r="O637">
+        <f>IF(L637="","",IF(M637="",L637,L637*(1-M637)))</f>
+        <v/>
+      </c>
+      <c r="R637" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="n">
+        <v>646</v>
+      </c>
+      <c r="B638" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C638">
+        <f>IF(B638="","",TEXT(B638,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>5 inch 7 feet wood × 4 pcs (gate frame, B unit)</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I638" t="n">
+        <v>2.916666666666667</v>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K638" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L638">
+        <f>IF(OR(I638="",K638=""),"",I638*K638)</f>
+        <v/>
+      </c>
+      <c r="N638">
+        <f>M638*L638</f>
+        <v/>
+      </c>
+      <c r="O638">
+        <f>IF(L638="","",IF(M638="",L638,L638*(1-M638)))</f>
+        <v/>
+      </c>
+      <c r="R638" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="n">
+        <v>647</v>
+      </c>
+      <c r="B639" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C639">
+        <f>IF(B639="","",TEXT(B639,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>4 inch 7 feet wood × 6 pcs (gate frame, B unit)</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I639" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K639" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L639">
+        <f>IF(OR(I639="",K639=""),"",I639*K639)</f>
+        <v/>
+      </c>
+      <c r="N639">
+        <f>M639*L639</f>
+        <v/>
+      </c>
+      <c r="O639">
+        <f>IF(L639="","",IF(M639="",L639,L639*(1-M639)))</f>
+        <v/>
+      </c>
+      <c r="R639" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="n">
+        <v>648</v>
+      </c>
+      <c r="B640" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C640">
+        <f>IF(B640="","",TEXT(B640,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>5 inch 3.5 feet wood × 2 pcs (gate frame, B unit)</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I640" t="n">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K640" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L640">
+        <f>IF(OR(I640="",K640=""),"",I640*K640)</f>
+        <v/>
+      </c>
+      <c r="N640">
+        <f>M640*L640</f>
+        <v/>
+      </c>
+      <c r="O640">
+        <f>IF(L640="","",IF(M640="",L640,L640*(1-M640)))</f>
+        <v/>
+      </c>
+      <c r="R640" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="n">
+        <v>649</v>
+      </c>
+      <c r="B641" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C641">
+        <f>IF(B641="","",TEXT(B641,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>4 inch 3.5 feet wood × 3 pcs (gate frame, B unit)</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I641" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>cft</t>
+        </is>
+      </c>
+      <c r="K641" t="n">
+        <v>3300</v>
+      </c>
+      <c r="L641">
+        <f>IF(OR(I641="",K641=""),"",I641*K641)</f>
+        <v/>
+      </c>
+      <c r="N641">
+        <f>M641*L641</f>
+        <v/>
+      </c>
+      <c r="O641">
+        <f>IF(L641="","",IF(M641="",L641,L641*(1-M641)))</f>
+        <v/>
+      </c>
+      <c r="R641" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="n">
+        <v>650</v>
+      </c>
+      <c r="B642" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C642">
+        <f>IF(B642="","",TEXT(B642,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>Labour (gate frame wood, B unit)</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="I642" t="n">
+        <v>1</v>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K642" t="n">
+        <v>400</v>
+      </c>
+      <c r="L642">
+        <f>IF(OR(I642="",K642=""),"",I642*K642)</f>
+        <v/>
+      </c>
+      <c r="N642">
+        <f>M642*L642</f>
+        <v/>
+      </c>
+      <c r="O642">
+        <f>IF(L642="","",IF(M642="",L642,L642*(1-M642)))</f>
+        <v/>
+      </c>
+      <c r="R642" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B633" s="60" t="n"/>
-      <c r="C633" s="60" t="n"/>
-      <c r="D633" s="60" t="n"/>
-      <c r="E633" s="60" t="n"/>
-      <c r="F633" s="60" t="n"/>
-      <c r="G633" s="60" t="n"/>
-      <c r="H633" s="60" t="n"/>
-      <c r="I633" s="60" t="n"/>
-      <c r="J633" s="60" t="n"/>
-      <c r="K633" s="60" t="n"/>
-      <c r="L633" s="61">
-        <f>SUM(L5:L632)</f>
-        <v/>
-      </c>
-      <c r="M633" s="60" t="n"/>
-      <c r="N633" s="60" t="n"/>
-      <c r="O633" s="61">
+      <c r="B643" s="60" t="n"/>
+      <c r="C643" s="60" t="n"/>
+      <c r="D643" s="60" t="n"/>
+      <c r="E643" s="60" t="n"/>
+      <c r="F643" s="60" t="n"/>
+      <c r="G643" s="60" t="n"/>
+      <c r="H643" s="60" t="n"/>
+      <c r="I643" s="60" t="n"/>
+      <c r="J643" s="60" t="n"/>
+      <c r="K643" s="60" t="n"/>
+      <c r="L643" s="61">
+        <f>SUM(L5:L642)</f>
+        <v/>
+      </c>
+      <c r="M643" s="60" t="n"/>
+      <c r="N643" s="60" t="n"/>
+      <c r="O643" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P633" s="60" t="n"/>
-      <c r="Q633" s="60" t="n"/>
+      <c r="P643" s="60" t="n"/>
+      <c r="Q643" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -48644,16 +49294,44 @@
       <c r="A103" s="41" t="n">
         <v>109</v>
       </c>
-      <c r="B103" s="45" t="n"/>
-      <c r="C103" s="47" t="n"/>
-      <c r="D103" s="47" t="n"/>
-      <c r="E103" s="47" t="n"/>
-      <c r="F103" s="47" t="n"/>
-      <c r="G103" s="62" t="n"/>
-      <c r="H103" s="47" t="n"/>
+      <c r="B103" s="45" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C103" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D103" s="47" t="inlineStr">
+        <is>
+          <t>Khutauna Chirai mill</t>
+        </is>
+      </c>
+      <c r="E103" s="47" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F103" s="47" t="inlineStr">
+        <is>
+          <t>Wood for gate frames — C unit ₹42,509 + B unit ₹26,869</t>
+        </is>
+      </c>
+      <c r="G103" s="62" t="n">
+        <v>69378</v>
+      </c>
+      <c r="H103" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I103" s="47" t="n"/>
       <c r="J103" s="47" t="n"/>
-      <c r="K103" s="47" t="n"/>
+      <c r="K103" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L103" s="50">
         <f>IF(G113="","",IF(L112="",G113,L112+G113))</f>
         <v/>

</xml_diff>

<commit_message>
Add: ₹70,000 paid to Pappu Hardware by Avinash (due now ₹7,353)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -49342,16 +49342,44 @@
       <c r="A104" s="43" t="n">
         <v>110</v>
       </c>
-      <c r="B104" s="53" t="n"/>
-      <c r="C104" s="55" t="n"/>
-      <c r="D104" s="55" t="n"/>
-      <c r="E104" s="55" t="n"/>
-      <c r="F104" s="55" t="n"/>
-      <c r="G104" s="63" t="n"/>
-      <c r="H104" s="55" t="n"/>
+      <c r="B104" s="53" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C104" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D104" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E104" s="55" t="inlineStr">
+        <is>
+          <t>Steel / Iron + Cement + Building Materials</t>
+        </is>
+      </c>
+      <c r="F104" s="55" t="inlineStr">
+        <is>
+          <t>Part payment against Oct bills</t>
+        </is>
+      </c>
+      <c r="G104" s="63" t="n">
+        <v>70000</v>
+      </c>
+      <c r="H104" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I104" s="55" t="n"/>
       <c r="J104" s="55" t="n"/>
-      <c r="K104" s="55" t="n"/>
+      <c r="K104" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L104" s="58">
         <f>IF(G114="","",IF(L113="",G114,L113+G114))</f>
         <v/>

</xml_diff>

<commit_message>
Add: Papa ₹25k (7-Oct) + ₹20k (8-Oct) to Econ Builder; Avinash ₹21,065 to Mittal Electric
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R643"/>
+  <dimension ref="A1:R646"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -32757,33 +32757,213 @@
       </c>
     </row>
     <row r="643">
-      <c r="A643" s="60" t="inlineStr">
+      <c r="A643" t="n">
+        <v>651</v>
+      </c>
+      <c r="B643" s="128" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C643">
+        <f>IF(B643="","",TEXT(B643,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>Construction work done — general site supervision &amp; labour (Papa, 7-Oct)</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I643" t="n">
+        <v>1</v>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K643" t="n">
+        <v>25000</v>
+      </c>
+      <c r="L643">
+        <f>IF(OR(I643="",K643=""),"",I643*K643)</f>
+        <v/>
+      </c>
+      <c r="N643">
+        <f>M643*L643</f>
+        <v/>
+      </c>
+      <c r="O643">
+        <f>IF(L643="","",IF(M643="",L643,L643*(1-M643)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="n">
+        <v>652</v>
+      </c>
+      <c r="B644" s="128" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C644">
+        <f>IF(B644="","",TEXT(B644,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Engineer Supervision</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>Construction work done — general site supervision &amp; labour (Papa, 8-Oct)</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I644" t="n">
+        <v>1</v>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K644" t="n">
+        <v>20000</v>
+      </c>
+      <c r="L644">
+        <f>IF(OR(I644="",K644=""),"",I644*K644)</f>
+        <v/>
+      </c>
+      <c r="N644">
+        <f>M644*L644</f>
+        <v/>
+      </c>
+      <c r="O644">
+        <f>IF(L644="","",IF(M644="",L644,L644*(1-M644)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="n">
+        <v>653</v>
+      </c>
+      <c r="B645" s="128" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C645">
+        <f>IF(B645="","",TEXT(B645,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>Electrical Items</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>Electrical items — Mittal Electric, Darbhanga</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>Mittal Electric</t>
+        </is>
+      </c>
+      <c r="I645" t="n">
+        <v>1</v>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K645" t="n">
+        <v>21065</v>
+      </c>
+      <c r="L645">
+        <f>IF(OR(I645="",K645=""),"",I645*K645)</f>
+        <v/>
+      </c>
+      <c r="N645">
+        <f>M645*L645</f>
+        <v/>
+      </c>
+      <c r="O645">
+        <f>IF(L645="","",IF(M645="",L645,L645*(1-M645)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B643" s="60" t="n"/>
-      <c r="C643" s="60" t="n"/>
-      <c r="D643" s="60" t="n"/>
-      <c r="E643" s="60" t="n"/>
-      <c r="F643" s="60" t="n"/>
-      <c r="G643" s="60" t="n"/>
-      <c r="H643" s="60" t="n"/>
-      <c r="I643" s="60" t="n"/>
-      <c r="J643" s="60" t="n"/>
-      <c r="K643" s="60" t="n"/>
-      <c r="L643" s="61">
-        <f>SUM(L5:L642)</f>
-        <v/>
-      </c>
-      <c r="M643" s="60" t="n"/>
-      <c r="N643" s="60" t="n"/>
-      <c r="O643" s="61">
+      <c r="B646" s="60" t="n"/>
+      <c r="C646" s="60" t="n"/>
+      <c r="D646" s="60" t="n"/>
+      <c r="E646" s="60" t="n"/>
+      <c r="F646" s="60" t="n"/>
+      <c r="G646" s="60" t="n"/>
+      <c r="H646" s="60" t="n"/>
+      <c r="I646" s="60" t="n"/>
+      <c r="J646" s="60" t="n"/>
+      <c r="K646" s="60" t="n"/>
+      <c r="L646" s="61">
+        <f>SUM(L5:L645)</f>
+        <v/>
+      </c>
+      <c r="M646" s="60" t="n"/>
+      <c r="N646" s="60" t="n"/>
+      <c r="O646" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P643" s="60" t="n"/>
-      <c r="Q643" s="60" t="n"/>
+      <c r="P646" s="60" t="n"/>
+      <c r="Q646" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -49390,16 +49570,44 @@
       <c r="A105" s="41" t="n">
         <v>111</v>
       </c>
-      <c r="B105" s="45" t="n"/>
-      <c r="C105" s="47" t="n"/>
-      <c r="D105" s="47" t="n"/>
-      <c r="E105" s="47" t="n"/>
-      <c r="F105" s="47" t="n"/>
-      <c r="G105" s="62" t="n"/>
-      <c r="H105" s="47" t="n"/>
+      <c r="B105" s="45" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C105" s="47" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D105" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E105" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F105" s="47" t="inlineStr">
+        <is>
+          <t>Construction work done — general (Papa, 7-Oct)</t>
+        </is>
+      </c>
+      <c r="G105" s="62" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H105" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I105" s="47" t="n"/>
       <c r="J105" s="47" t="n"/>
-      <c r="K105" s="47" t="n"/>
+      <c r="K105" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L105" s="50">
         <f>IF(G115="","",IF(L114="",G115,L114+G115))</f>
         <v/>
@@ -49410,16 +49618,44 @@
       <c r="A106" s="43" t="n">
         <v>112</v>
       </c>
-      <c r="B106" s="53" t="n"/>
-      <c r="C106" s="55" t="n"/>
-      <c r="D106" s="55" t="n"/>
-      <c r="E106" s="55" t="n"/>
-      <c r="F106" s="55" t="n"/>
-      <c r="G106" s="63" t="n"/>
-      <c r="H106" s="55" t="n"/>
+      <c r="B106" s="53" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C106" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D106" s="55" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E106" s="55" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F106" s="55" t="inlineStr">
+        <is>
+          <t>Construction work done — general (Papa, 8-Oct)</t>
+        </is>
+      </c>
+      <c r="G106" s="63" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H106" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I106" s="55" t="n"/>
       <c r="J106" s="55" t="n"/>
-      <c r="K106" s="55" t="n"/>
+      <c r="K106" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L106" s="58">
         <f>IF(G116="","",IF(L115="",G116,L115+G116))</f>
         <v/>
@@ -49430,16 +49666,44 @@
       <c r="A107" s="41" t="n">
         <v>113</v>
       </c>
-      <c r="B107" s="45" t="n"/>
-      <c r="C107" s="47" t="n"/>
-      <c r="D107" s="47" t="n"/>
-      <c r="E107" s="47" t="n"/>
-      <c r="F107" s="47" t="n"/>
-      <c r="G107" s="62" t="n"/>
-      <c r="H107" s="47" t="n"/>
+      <c r="B107" s="45" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C107" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D107" s="47" t="inlineStr">
+        <is>
+          <t>Mittal Electric</t>
+        </is>
+      </c>
+      <c r="E107" s="47" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F107" s="47" t="inlineStr">
+        <is>
+          <t>Electrical items — Mittal Electric, Darbhanga</t>
+        </is>
+      </c>
+      <c r="G107" s="62" t="n">
+        <v>21065</v>
+      </c>
+      <c r="H107" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I107" s="47" t="n"/>
       <c r="J107" s="47" t="n"/>
-      <c r="K107" s="47" t="n"/>
+      <c r="K107" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L107" s="50">
         <f>IF(G117="","",IF(L116="",G117,L116+G117))</f>
         <v/>

</xml_diff>

<commit_message>
Add: sand 40 MT ₹56,000 (Sand Truck Wala) and diesel 10 L ₹1,000, paid by Avinash 9-Oct
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -6539,7 +6539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R646"/>
+  <dimension ref="A1:R648"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -32937,33 +32937,153 @@
       </c>
     </row>
     <row r="646">
-      <c r="A646" s="60" t="inlineStr">
+      <c r="A646" t="n">
+        <v>654</v>
+      </c>
+      <c r="B646" s="128" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C646">
+        <f>IF(B646="","",TEXT(B646,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>Sand delivery — 40 MT @ ₹1,400/MT</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="I646" t="n">
+        <v>40</v>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="K646" t="n">
+        <v>1400</v>
+      </c>
+      <c r="L646">
+        <f>IF(OR(I646="",K646=""),"",I646*K646)</f>
+        <v/>
+      </c>
+      <c r="N646">
+        <f>M646*L646</f>
+        <v/>
+      </c>
+      <c r="O646">
+        <f>IF(L646="","",IF(M646="",L646,L646*(1-M646)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="n">
+        <v>655</v>
+      </c>
+      <c r="B647" s="128" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C647">
+        <f>IF(B647="","",TEXT(B647,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>Diesel 10 litres @ ₹100/L</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I647" t="n">
+        <v>10</v>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>Litres</t>
+        </is>
+      </c>
+      <c r="K647" t="n">
+        <v>100</v>
+      </c>
+      <c r="L647">
+        <f>IF(OR(I647="",K647=""),"",I647*K647)</f>
+        <v/>
+      </c>
+      <c r="N647">
+        <f>M647*L647</f>
+        <v/>
+      </c>
+      <c r="O647">
+        <f>IF(L647="","",IF(M647="",L647,L647*(1-M647)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B646" s="60" t="n"/>
-      <c r="C646" s="60" t="n"/>
-      <c r="D646" s="60" t="n"/>
-      <c r="E646" s="60" t="n"/>
-      <c r="F646" s="60" t="n"/>
-      <c r="G646" s="60" t="n"/>
-      <c r="H646" s="60" t="n"/>
-      <c r="I646" s="60" t="n"/>
-      <c r="J646" s="60" t="n"/>
-      <c r="K646" s="60" t="n"/>
-      <c r="L646" s="61">
-        <f>SUM(L5:L645)</f>
-        <v/>
-      </c>
-      <c r="M646" s="60" t="n"/>
-      <c r="N646" s="60" t="n"/>
-      <c r="O646" s="61">
+      <c r="B648" s="60" t="n"/>
+      <c r="C648" s="60" t="n"/>
+      <c r="D648" s="60" t="n"/>
+      <c r="E648" s="60" t="n"/>
+      <c r="F648" s="60" t="n"/>
+      <c r="G648" s="60" t="n"/>
+      <c r="H648" s="60" t="n"/>
+      <c r="I648" s="60" t="n"/>
+      <c r="J648" s="60" t="n"/>
+      <c r="K648" s="60" t="n"/>
+      <c r="L648" s="61">
+        <f>SUM(L5:L647)</f>
+        <v/>
+      </c>
+      <c r="M648" s="60" t="n"/>
+      <c r="N648" s="60" t="n"/>
+      <c r="O648" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P646" s="60" t="n"/>
-      <c r="Q646" s="60" t="n"/>
+      <c r="P648" s="60" t="n"/>
+      <c r="Q648" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -49714,16 +49834,44 @@
       <c r="A108" s="43" t="n">
         <v>114</v>
       </c>
-      <c r="B108" s="53" t="n"/>
-      <c r="C108" s="55" t="n"/>
-      <c r="D108" s="55" t="n"/>
-      <c r="E108" s="55" t="n"/>
-      <c r="F108" s="55" t="n"/>
-      <c r="G108" s="63" t="n"/>
-      <c r="H108" s="55" t="n"/>
+      <c r="B108" s="53" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C108" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D108" s="55" t="inlineStr">
+        <is>
+          <t>Sand Truck Wala</t>
+        </is>
+      </c>
+      <c r="E108" s="55" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F108" s="55" t="inlineStr">
+        <is>
+          <t>Sand delivery — 40 MT</t>
+        </is>
+      </c>
+      <c r="G108" s="63" t="n">
+        <v>56000</v>
+      </c>
+      <c r="H108" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I108" s="55" t="n"/>
       <c r="J108" s="55" t="n"/>
-      <c r="K108" s="55" t="n"/>
+      <c r="K108" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L108" s="58">
         <f>IF(G118="","",IF(L117="",G118,L117+G118))</f>
         <v/>
@@ -49734,16 +49882,44 @@
       <c r="A109" s="41" t="n">
         <v>115</v>
       </c>
-      <c r="B109" s="45" t="n"/>
-      <c r="C109" s="47" t="n"/>
-      <c r="D109" s="47" t="n"/>
-      <c r="E109" s="47" t="n"/>
-      <c r="F109" s="47" t="n"/>
-      <c r="G109" s="62" t="n"/>
-      <c r="H109" s="47" t="n"/>
+      <c r="B109" s="45" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C109" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D109" s="47" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="E109" s="47" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F109" s="47" t="inlineStr">
+        <is>
+          <t>Diesel 10 litres</t>
+        </is>
+      </c>
+      <c r="G109" s="62" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H109" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I109" s="47" t="n"/>
       <c r="J109" s="47" t="n"/>
-      <c r="K109" s="47" t="n"/>
+      <c r="K109" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L109" s="50">
         <f>IF(G119="","",IF(L118="",G119,L118+G119))</f>
         <v/>

</xml_diff>

<commit_message>
Count all Econ Builder amounts under Professional Fees (₹7,16,000)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -2465,7 +2465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="99" min="1" max="1"/>
@@ -2907,30 +2907,30 @@
       <c r="I16" s="82" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="99">
-      <c r="A17" s="74" t="inlineStr">
+      <c r="A17" s="77" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="84">
+      <c r="B17" s="87">
         <f>SUM(B5:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="84">
+      <c r="C17" s="87">
         <f>SUM(C5:C16)</f>
         <v/>
       </c>
-      <c r="D17" s="84">
+      <c r="D17" s="87">
         <f>SUM(D5:D16)</f>
         <v/>
       </c>
-      <c r="E17" s="96">
+      <c r="E17" s="97">
         <f>C17-D17</f>
         <v/>
       </c>
-      <c r="F17" s="85" t="n"/>
-      <c r="G17" s="86" t="n"/>
-      <c r="H17" s="74" t="n"/>
+      <c r="F17" s="89" t="n"/>
+      <c r="G17" s="90" t="n"/>
+      <c r="H17" s="77" t="n"/>
       <c r="I17" s="82" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="99">
@@ -3010,6 +3010,21 @@
       <c r="H24" s="82" t="n"/>
       <c r="I24" s="82" t="n"/>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -5115,7 +5130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
@@ -6605,6 +6620,17 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
@@ -6622,7 +6648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R699"/>
+  <dimension ref="A1:R648"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -27767,7 +27793,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>Transport · Food · Misc</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F559" t="inlineStr">
@@ -27827,7 +27853,7 @@
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -27887,7 +27913,7 @@
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F561" t="inlineStr">
@@ -27947,7 +27973,7 @@
       </c>
       <c r="E562" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F562" t="inlineStr">
@@ -28007,7 +28033,7 @@
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F563" t="inlineStr">
@@ -28067,7 +28093,7 @@
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F564" t="inlineStr">
@@ -28127,7 +28153,7 @@
       </c>
       <c r="E565" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F565" t="inlineStr">
@@ -28187,7 +28213,7 @@
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -28247,7 +28273,7 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -28307,7 +28333,7 @@
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F568" t="inlineStr">
@@ -28367,7 +28393,7 @@
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F569" t="inlineStr">
@@ -28427,7 +28453,7 @@
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F570" t="inlineStr">
@@ -28487,7 +28513,7 @@
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F571" t="inlineStr">
@@ -28547,7 +28573,7 @@
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F572" t="inlineStr">
@@ -28607,7 +28633,7 @@
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F573" t="inlineStr">
@@ -28667,7 +28693,7 @@
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F574" t="inlineStr">
@@ -28727,7 +28753,7 @@
       </c>
       <c r="E575" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F575" t="inlineStr">
@@ -28787,7 +28813,7 @@
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F576" t="inlineStr">
@@ -28847,7 +28873,7 @@
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F577" t="inlineStr">
@@ -28907,7 +28933,7 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F578" t="inlineStr">
@@ -28967,7 +28993,7 @@
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>Transport · Food · Misc</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F579" t="inlineStr">
@@ -29027,7 +29053,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F580" t="inlineStr">
@@ -29087,7 +29113,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F581" t="inlineStr">
@@ -29147,7 +29173,7 @@
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -29207,7 +29233,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F583" t="inlineStr">
@@ -29267,7 +29293,7 @@
       </c>
       <c r="E584" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F584" t="inlineStr">
@@ -29327,7 +29353,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -29387,7 +29413,7 @@
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F586" t="inlineStr">
@@ -29447,7 +29473,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F587" t="inlineStr">
@@ -29507,7 +29533,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F588" t="inlineStr">
@@ -29567,7 +29593,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F589" t="inlineStr">
@@ -29627,7 +29653,7 @@
       </c>
       <c r="E590" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F590" t="inlineStr">
@@ -29687,7 +29713,7 @@
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
@@ -29747,7 +29773,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F592" t="inlineStr">
@@ -29807,7 +29833,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>Transport · Food · Misc</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F593" t="inlineStr">
@@ -29867,7 +29893,7 @@
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F594" t="inlineStr">
@@ -29927,7 +29953,7 @@
       </c>
       <c r="E595" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F595" t="inlineStr">
@@ -29987,7 +30013,7 @@
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F596" t="inlineStr">
@@ -30047,7 +30073,7 @@
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F597" t="inlineStr">
@@ -30107,7 +30133,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F598" t="inlineStr">
@@ -30167,7 +30193,7 @@
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F599" t="inlineStr">
@@ -30227,7 +30253,7 @@
       </c>
       <c r="E600" t="inlineStr">
         <is>
-          <t>Labour</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F600" t="inlineStr">
@@ -30407,7 +30433,7 @@
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>Transport · Food · Misc</t>
+          <t>Professional Fees</t>
         </is>
       </c>
       <c r="F603" t="inlineStr">
@@ -33168,57 +33194,6 @@
       <c r="P648" s="60" t="n"/>
       <c r="Q648" s="60" t="n"/>
     </row>
-    <row r="649"/>
-    <row r="650"/>
-    <row r="651"/>
-    <row r="652"/>
-    <row r="653"/>
-    <row r="654"/>
-    <row r="655"/>
-    <row r="656"/>
-    <row r="657"/>
-    <row r="658"/>
-    <row r="659"/>
-    <row r="660"/>
-    <row r="661"/>
-    <row r="662"/>
-    <row r="663"/>
-    <row r="664"/>
-    <row r="665"/>
-    <row r="666"/>
-    <row r="667"/>
-    <row r="668"/>
-    <row r="669"/>
-    <row r="670"/>
-    <row r="671"/>
-    <row r="672"/>
-    <row r="673"/>
-    <row r="674"/>
-    <row r="675"/>
-    <row r="676"/>
-    <row r="677"/>
-    <row r="678"/>
-    <row r="679"/>
-    <row r="680"/>
-    <row r="681"/>
-    <row r="682"/>
-    <row r="683"/>
-    <row r="684"/>
-    <row r="685"/>
-    <row r="686"/>
-    <row r="687"/>
-    <row r="688"/>
-    <row r="689"/>
-    <row r="690"/>
-    <row r="691"/>
-    <row r="692"/>
-    <row r="693"/>
-    <row r="694"/>
-    <row r="695"/>
-    <row r="696"/>
-    <row r="697"/>
-    <row r="698"/>
-    <row r="699"/>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
   <mergeCells count="2">
@@ -58422,12 +58397,12 @@
     <row r="14" ht="15.75" customHeight="1" s="99">
       <c r="A14" s="44" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="B14" s="44" t="inlineStr">
         <is>
-          <t>Fabrication</t>
+          <t>Electrical Items</t>
         </is>
       </c>
       <c r="C14" s="69">
@@ -58463,12 +58438,12 @@
     <row r="15" ht="15.75" customHeight="1" s="99">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Building Materials</t>
         </is>
       </c>
       <c r="B15" s="42" t="inlineStr">
         <is>
-          <t>Electrical Items</t>
+          <t>Dr Fixit</t>
         </is>
       </c>
       <c r="C15" s="64">
@@ -58477,7 +58452,7 @@
       </c>
       <c r="D15" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>litres</t>
         </is>
       </c>
       <c r="E15" s="65">
@@ -58504,12 +58479,12 @@
     <row r="16" ht="15.75" customHeight="1" s="99">
       <c r="A16" s="44" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>Steel / Iron</t>
         </is>
       </c>
       <c r="B16" s="44" t="inlineStr">
         <is>
-          <t>Dr Fixit</t>
+          <t>Tiscon 16mm</t>
         </is>
       </c>
       <c r="C16" s="69">
@@ -58518,7 +58493,7 @@
       </c>
       <c r="D16" s="44" t="inlineStr">
         <is>
-          <t>litres</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="E16" s="70">
@@ -58550,7 +58525,7 @@
       </c>
       <c r="B17" s="42" t="inlineStr">
         <is>
-          <t>Water Tank</t>
+          <t>Binding Wire</t>
         </is>
       </c>
       <c r="C17" s="64">
@@ -58559,7 +58534,7 @@
       </c>
       <c r="D17" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E17" s="65">
@@ -58591,7 +58566,7 @@
       </c>
       <c r="B18" s="44" t="inlineStr">
         <is>
-          <t>Tiscon 16mm</t>
+          <t>Wire</t>
         </is>
       </c>
       <c r="C18" s="69">
@@ -58600,7 +58575,7 @@
       </c>
       <c r="D18" s="44" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="E18" s="70">
@@ -58627,12 +58602,12 @@
     <row r="19" ht="15.75" customHeight="1" s="99">
       <c r="A19" s="42" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>Steel / Iron</t>
         </is>
       </c>
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>Binding Wire</t>
+          <t>Rings</t>
         </is>
       </c>
       <c r="C19" s="64">
@@ -58641,7 +58616,7 @@
       </c>
       <c r="D19" s="42" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E19" s="65">
@@ -58668,12 +58643,12 @@
     <row r="20" ht="15.75" customHeight="1" s="99">
       <c r="A20" s="44" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Building Materials</t>
         </is>
       </c>
       <c r="B20" s="44" t="inlineStr">
         <is>
-          <t>Wire</t>
+          <t>Cover Block</t>
         </is>
       </c>
       <c r="C20" s="69">
@@ -58682,7 +58657,7 @@
       </c>
       <c r="D20" s="44" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="E20" s="70">
@@ -58709,12 +58684,12 @@
     <row r="21" ht="15.75" customHeight="1" s="99">
       <c r="A21" s="42" t="inlineStr">
         <is>
-          <t>Steel / Iron</t>
+          <t>Building Materials</t>
         </is>
       </c>
       <c r="B21" s="42" t="inlineStr">
         <is>
-          <t>Rings</t>
+          <t>Nails</t>
         </is>
       </c>
       <c r="C21" s="64">
@@ -58723,7 +58698,7 @@
       </c>
       <c r="D21" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>bags</t>
         </is>
       </c>
       <c r="E21" s="65">
@@ -58755,7 +58730,7 @@
       </c>
       <c r="B22" s="44" t="inlineStr">
         <is>
-          <t>Cover Block</t>
+          <t>Chemical</t>
         </is>
       </c>
       <c r="C22" s="69">
@@ -58764,7 +58739,7 @@
       </c>
       <c r="D22" s="44" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>litres</t>
         </is>
       </c>
       <c r="E22" s="70">
@@ -58796,7 +58771,7 @@
       </c>
       <c r="B23" s="42" t="inlineStr">
         <is>
-          <t>Nails</t>
+          <t>Wire</t>
         </is>
       </c>
       <c r="C23" s="64">
@@ -58805,7 +58780,7 @@
       </c>
       <c r="D23" s="42" t="inlineStr">
         <is>
-          <t>bags</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E23" s="65">
@@ -58837,7 +58812,7 @@
       </c>
       <c r="B24" s="44" t="inlineStr">
         <is>
-          <t>Chemical</t>
+          <t>Material Transport</t>
         </is>
       </c>
       <c r="C24" s="69">
@@ -58846,7 +58821,7 @@
       </c>
       <c r="D24" s="44" t="inlineStr">
         <is>
-          <t>litres</t>
+          <t>trips</t>
         </is>
       </c>
       <c r="E24" s="70">
@@ -58871,127 +58846,37 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="99">
-      <c r="A25" s="42" t="inlineStr">
-        <is>
-          <t>Building Materials</t>
-        </is>
-      </c>
-      <c r="B25" s="42" t="inlineStr">
-        <is>
-          <t>Wire</t>
-        </is>
-      </c>
-      <c r="C25" s="64">
-        <f>SUMIFS('All Transactions'!I:I,'All Transactions'!E:E,A25,'All Transactions'!F:F,B25,'All Transactions'!J:J,"&lt;&gt;Lumpsum",'All Transactions'!J:J,"&lt;&gt;Service",'All Transactions'!J:J,"&lt;&gt;Lot",'All Transactions'!J:J,"&lt;&gt;Advance")</f>
-        <v/>
-      </c>
-      <c r="D25" s="42" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E25" s="65">
-        <f>IFERROR(IF(C25=0,"",F25/C25),"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="66">
-        <f>SUMIFS('All Transactions'!L:L,'All Transactions'!E:E,A25,'All Transactions'!F:F,B25)</f>
-        <v/>
-      </c>
-      <c r="G25" s="67">
-        <f>F25-H25</f>
-        <v/>
-      </c>
-      <c r="H25" s="66">
-        <f>SUMIFS('All Transactions'!O:O,'All Transactions'!E:E,A25,'All Transactions'!F:F,B25)</f>
-        <v/>
-      </c>
-      <c r="I25" s="68">
-        <f>IFERROR(H25/H$35,"")</f>
-        <v/>
-      </c>
+      <c r="A25" s="42" t="n"/>
+      <c r="B25" s="42" t="n"/>
+      <c r="C25" s="64" t="n"/>
+      <c r="D25" s="42" t="n"/>
+      <c r="E25" s="65" t="n"/>
+      <c r="F25" s="66" t="n"/>
+      <c r="G25" s="67" t="n"/>
+      <c r="H25" s="66" t="n"/>
+      <c r="I25" s="68" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="99">
-      <c r="A26" s="44" t="inlineStr">
-        <is>
-          <t>Building Materials</t>
-        </is>
-      </c>
-      <c r="B26" s="44" t="inlineStr">
-        <is>
-          <t>Plywood/Shuttering</t>
-        </is>
-      </c>
-      <c r="C26" s="69">
-        <f>SUMIFS('All Transactions'!I:I,'All Transactions'!E:E,A26,'All Transactions'!F:F,B26,'All Transactions'!J:J,"&lt;&gt;Lumpsum",'All Transactions'!J:J,"&lt;&gt;Service",'All Transactions'!J:J,"&lt;&gt;Lot",'All Transactions'!J:J,"&lt;&gt;Advance")</f>
-        <v/>
-      </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="70">
-        <f>IFERROR(IF(C26=0,"",F26/C26),"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="71">
-        <f>SUMIFS('All Transactions'!L:L,'All Transactions'!E:E,A26,'All Transactions'!F:F,B26)</f>
-        <v/>
-      </c>
-      <c r="G26" s="72">
-        <f>F26-H26</f>
-        <v/>
-      </c>
-      <c r="H26" s="71">
-        <f>SUMIFS('All Transactions'!O:O,'All Transactions'!E:E,A26,'All Transactions'!F:F,B26)</f>
-        <v/>
-      </c>
-      <c r="I26" s="73">
-        <f>IFERROR(H26/H$35,"")</f>
-        <v/>
-      </c>
+      <c r="A26" s="44" t="n"/>
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="69" t="n"/>
+      <c r="D26" s="44" t="n"/>
+      <c r="E26" s="70" t="n"/>
+      <c r="F26" s="71" t="n"/>
+      <c r="G26" s="72" t="n"/>
+      <c r="H26" s="71" t="n"/>
+      <c r="I26" s="73" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="99">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>Building Materials</t>
-        </is>
-      </c>
-      <c r="B27" s="42" t="inlineStr">
-        <is>
-          <t>Material Transport</t>
-        </is>
-      </c>
-      <c r="C27" s="64">
-        <f>SUMIFS('All Transactions'!I:I,'All Transactions'!E:E,A27,'All Transactions'!F:F,B27,'All Transactions'!J:J,"&lt;&gt;Lumpsum",'All Transactions'!J:J,"&lt;&gt;Service",'All Transactions'!J:J,"&lt;&gt;Lot",'All Transactions'!J:J,"&lt;&gt;Advance")</f>
-        <v/>
-      </c>
-      <c r="D27" s="42" t="inlineStr">
-        <is>
-          <t>trips</t>
-        </is>
-      </c>
-      <c r="E27" s="65">
-        <f>IFERROR(IF(C27=0,"",F27/C27),"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="66">
-        <f>SUMIFS('All Transactions'!L:L,'All Transactions'!E:E,A27,'All Transactions'!F:F,B27)</f>
-        <v/>
-      </c>
-      <c r="G27" s="67">
-        <f>F27-H27</f>
-        <v/>
-      </c>
-      <c r="H27" s="66">
-        <f>SUMIFS('All Transactions'!O:O,'All Transactions'!E:E,A27,'All Transactions'!F:F,B27)</f>
-        <v/>
-      </c>
-      <c r="I27" s="68">
-        <f>IFERROR(H27/H$35,"")</f>
-        <v/>
-      </c>
+      <c r="A27" s="42" t="n"/>
+      <c r="B27" s="42" t="n"/>
+      <c r="C27" s="64" t="n"/>
+      <c r="D27" s="42" t="n"/>
+      <c r="E27" s="65" t="n"/>
+      <c r="F27" s="66" t="n"/>
+      <c r="G27" s="67" t="n"/>
+      <c r="H27" s="66" t="n"/>
+      <c r="I27" s="68" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="99">
       <c r="A28" s="44" t="n"/>
@@ -67785,7 +67670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
@@ -68772,6 +68657,36 @@
       <c r="J29" s="74" t="n"/>
       <c r="K29" s="74" t="n"/>
     </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>

</xml_diff>

<commit_message>
Add: Pappu Hardware 13-Oct bill ₹1,42,843 (steel, gitti, cement, wire), paid by Avinash
Also untrack Excel lock file.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -2465,7 +2465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="99" min="1" max="1"/>
@@ -3010,21 +3010,6 @@
       <c r="H24" s="82" t="n"/>
       <c r="I24" s="82" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -5130,7 +5115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="99" min="1" max="1"/>
@@ -6620,17 +6605,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
@@ -6648,7 +6622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R648"/>
+  <dimension ref="A1:R659"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -33166,33 +33140,693 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="60" t="inlineStr">
+      <c r="A648" t="n">
+        <v>656</v>
+      </c>
+      <c r="B648" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C648">
+        <f>IF(B648="","",TEXT(B648,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>Tiscon 12mm rod 6 pcs</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I648" t="n">
+        <v>6</v>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K648" t="n">
+        <v>902</v>
+      </c>
+      <c r="L648">
+        <f>IF(OR(I648="",K648=""),"",I648*K648)</f>
+        <v/>
+      </c>
+      <c r="N648">
+        <f>M648*L648</f>
+        <v/>
+      </c>
+      <c r="O648">
+        <f>IF(L648="","",IF(M648="",L648,L648*(1-M648)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>657</v>
+      </c>
+      <c r="B649" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C649">
+        <f>IF(B649="","",TEXT(B649,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H649" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I649" t="n">
+        <v>1</v>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K649" t="n">
+        <v>350</v>
+      </c>
+      <c r="L649">
+        <f>IF(OR(I649="",K649=""),"",I649*K649)</f>
+        <v/>
+      </c>
+      <c r="N649">
+        <f>M649*L649</f>
+        <v/>
+      </c>
+      <c r="O649">
+        <f>IF(L649="","",IF(M649="",L649,L649*(1-M649)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>658</v>
+      </c>
+      <c r="B650" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C650">
+        <f>IF(B650="","",TEXT(B650,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>Binding Wire</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>Binding wire 60 kg @ ₹110</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I650" t="n">
+        <v>60</v>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="K650" t="n">
+        <v>110</v>
+      </c>
+      <c r="L650">
+        <f>IF(OR(I650="",K650=""),"",I650*K650)</f>
+        <v/>
+      </c>
+      <c r="N650">
+        <f>M650*L650</f>
+        <v/>
+      </c>
+      <c r="O650">
+        <f>IF(L650="","",IF(M650="",L650,L650*(1-M650)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>659</v>
+      </c>
+      <c r="B651" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C651">
+        <f>IF(B651="","",TEXT(B651,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm rod 32 pcs</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I651" t="n">
+        <v>32</v>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K651" t="n">
+        <v>620.5</v>
+      </c>
+      <c r="L651">
+        <f>IF(OR(I651="",K651=""),"",I651*K651)</f>
+        <v/>
+      </c>
+      <c r="N651">
+        <f>M651*L651</f>
+        <v/>
+      </c>
+      <c r="O651">
+        <f>IF(L651="","",IF(M651="",L651,L651*(1-M651)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>660</v>
+      </c>
+      <c r="B652" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C652">
+        <f>IF(B652="","",TEXT(B652,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm rod 84 pcs</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I652" t="n">
+        <v>84</v>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K652" t="n">
+        <v>405.297619047619</v>
+      </c>
+      <c r="L652">
+        <f>IF(OR(I652="",K652=""),"",I652*K652)</f>
+        <v/>
+      </c>
+      <c r="N652">
+        <f>M652*L652</f>
+        <v/>
+      </c>
+      <c r="O652">
+        <f>IF(L652="","",IF(M652="",L652,L652*(1-M652)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>661</v>
+      </c>
+      <c r="B653" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C653">
+        <f>IF(B653="","",TEXT(B653,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>Tiscon 8mm rod 24 pcs</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I653" t="n">
+        <v>24</v>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K653" t="n">
+        <v>404.1666666666667</v>
+      </c>
+      <c r="L653">
+        <f>IF(OR(I653="",K653=""),"",I653*K653)</f>
+        <v/>
+      </c>
+      <c r="N653">
+        <f>M653*L653</f>
+        <v/>
+      </c>
+      <c r="O653">
+        <f>IF(L653="","",IF(M653="",L653,L653*(1-M653)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>662</v>
+      </c>
+      <c r="B654" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C654">
+        <f>IF(B654="","",TEXT(B654,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Nails</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>Nails</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I654" t="n">
+        <v>1</v>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K654" t="n">
+        <v>150</v>
+      </c>
+      <c r="L654">
+        <f>IF(OR(I654="",K654=""),"",I654*K654)</f>
+        <v/>
+      </c>
+      <c r="N654">
+        <f>M654*L654</f>
+        <v/>
+      </c>
+      <c r="O654">
+        <f>IF(L654="","",IF(M654="",L654,L654*(1-M654)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>663</v>
+      </c>
+      <c r="B655" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C655">
+        <f>IF(B655="","",TEXT(B655,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>Steel / Iron</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>Tiscon 10mm rod 3 pcs</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I655" t="n">
+        <v>3</v>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="K655" t="n">
+        <v>610</v>
+      </c>
+      <c r="L655">
+        <f>IF(OR(I655="",K655=""),"",I655*K655)</f>
+        <v/>
+      </c>
+      <c r="N655">
+        <f>M655*L655</f>
+        <v/>
+      </c>
+      <c r="O655">
+        <f>IF(L655="","",IF(M655="",L655,L655*(1-M655)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>664</v>
+      </c>
+      <c r="B656" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C656">
+        <f>IF(B656="","",TEXT(B656,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>Concrete/Gitti</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>Gitti 4 trailers @ ₹9,500</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I656" t="n">
+        <v>4</v>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>Trailer</t>
+        </is>
+      </c>
+      <c r="K656" t="n">
+        <v>9500</v>
+      </c>
+      <c r="L656">
+        <f>IF(OR(I656="",K656=""),"",I656*K656)</f>
+        <v/>
+      </c>
+      <c r="N656">
+        <f>M656*L656</f>
+        <v/>
+      </c>
+      <c r="O656">
+        <f>IF(L656="","",IF(M656="",L656,L656*(1-M656)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>665</v>
+      </c>
+      <c r="B657" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C657">
+        <f>IF(B657="","",TEXT(B657,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>Concreto Uno cement 65 bags @ ₹380</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I657" t="n">
+        <v>65</v>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>Bag</t>
+        </is>
+      </c>
+      <c r="K657" t="n">
+        <v>380</v>
+      </c>
+      <c r="L657">
+        <f>IF(OR(I657="",K657=""),"",I657*K657)</f>
+        <v/>
+      </c>
+      <c r="N657">
+        <f>M657*L657</f>
+        <v/>
+      </c>
+      <c r="O657">
+        <f>IF(L657="","",IF(M657="",L657,L657*(1-M657)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>666</v>
+      </c>
+      <c r="B658" s="128" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C658">
+        <f>IF(B658="","",TEXT(B658,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Site Labour</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="I658" t="n">
+        <v>1</v>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K658" t="n">
+        <v>2200</v>
+      </c>
+      <c r="L658">
+        <f>IF(OR(I658="",K658=""),"",I658*K658)</f>
+        <v/>
+      </c>
+      <c r="N658">
+        <f>M658*L658</f>
+        <v/>
+      </c>
+      <c r="O658">
+        <f>IF(L658="","",IF(M658="",L658,L658*(1-M658)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B648" s="60" t="n"/>
-      <c r="C648" s="60" t="n"/>
-      <c r="D648" s="60" t="n"/>
-      <c r="E648" s="60" t="n"/>
-      <c r="F648" s="60" t="n"/>
-      <c r="G648" s="60" t="n"/>
-      <c r="H648" s="60" t="n"/>
-      <c r="I648" s="60" t="n"/>
-      <c r="J648" s="60" t="n"/>
-      <c r="K648" s="60" t="n"/>
-      <c r="L648" s="61">
-        <f>SUM(L5:L647)</f>
-        <v/>
-      </c>
-      <c r="M648" s="60" t="n"/>
-      <c r="N648" s="60" t="n"/>
-      <c r="O648" s="61">
+      <c r="B659" s="60" t="n"/>
+      <c r="C659" s="60" t="n"/>
+      <c r="D659" s="60" t="n"/>
+      <c r="E659" s="60" t="n"/>
+      <c r="F659" s="60" t="n"/>
+      <c r="G659" s="60" t="n"/>
+      <c r="H659" s="60" t="n"/>
+      <c r="I659" s="60" t="n"/>
+      <c r="J659" s="60" t="n"/>
+      <c r="K659" s="60" t="n"/>
+      <c r="L659" s="61">
+        <f>SUM(L5:L658)</f>
+        <v/>
+      </c>
+      <c r="M659" s="60" t="n"/>
+      <c r="N659" s="60" t="n"/>
+      <c r="O659" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P648" s="60" t="n"/>
-      <c r="Q648" s="60" t="n"/>
+      <c r="P659" s="60" t="n"/>
+      <c r="Q659" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -50195,16 +50829,44 @@
       <c r="A110" s="43" t="n">
         <v>116</v>
       </c>
-      <c r="B110" s="53" t="n"/>
-      <c r="C110" s="55" t="n"/>
-      <c r="D110" s="55" t="n"/>
-      <c r="E110" s="55" t="n"/>
-      <c r="F110" s="55" t="n"/>
-      <c r="G110" s="63" t="n"/>
-      <c r="H110" s="55" t="n"/>
+      <c r="B110" s="53" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C110" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D110" s="55" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E110" s="55" t="inlineStr">
+        <is>
+          <t>Steel / Iron + Cement + Building Materials</t>
+        </is>
+      </c>
+      <c r="F110" s="55" t="inlineStr">
+        <is>
+          <t>Full payment — 13-Oct bill (₹1,42,843)</t>
+        </is>
+      </c>
+      <c r="G110" s="63" t="n">
+        <v>142843</v>
+      </c>
+      <c r="H110" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I110" s="55" t="n"/>
       <c r="J110" s="55" t="n"/>
-      <c r="K110" s="55" t="n"/>
+      <c r="K110" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L110" s="58">
         <f>IF(G110="","",IF(L109="",G110,L109+G110))</f>
         <v/>
@@ -67670,7 +68332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="99" min="1" max="1"/>
@@ -68657,36 +69319,6 @@
       <c r="J29" s="74" t="n"/>
       <c r="K29" s="74" t="n"/>
     </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>

</xml_diff>

<commit_message>
Add: ₹7,353 paid to Pappu Hardware (Avinash, 14-Oct) — balance settled
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -50877,16 +50877,44 @@
       <c r="A111" s="41" t="n">
         <v>117</v>
       </c>
-      <c r="B111" s="45" t="n"/>
-      <c r="C111" s="47" t="n"/>
-      <c r="D111" s="47" t="n"/>
-      <c r="E111" s="47" t="n"/>
-      <c r="F111" s="47" t="n"/>
-      <c r="G111" s="62" t="n"/>
-      <c r="H111" s="47" t="n"/>
+      <c r="B111" s="45" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C111" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D111" s="47" t="inlineStr">
+        <is>
+          <t>Pappu Hardware</t>
+        </is>
+      </c>
+      <c r="E111" s="47" t="inlineStr">
+        <is>
+          <t>Steel / Iron + Cement + Building Materials</t>
+        </is>
+      </c>
+      <c r="F111" s="47" t="inlineStr">
+        <is>
+          <t>Balance settled — Oct bills</t>
+        </is>
+      </c>
+      <c r="G111" s="62" t="n">
+        <v>7353</v>
+      </c>
+      <c r="H111" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I111" s="47" t="n"/>
       <c r="J111" s="47" t="n"/>
-      <c r="K111" s="47" t="n"/>
+      <c r="K111" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L111" s="50">
         <f>IF(G111="","",IF(L110="",G111,L110+G111))</f>
         <v/>

</xml_diff>

<commit_message>
Add: 14-Oct entries — Econ Builder ₹30k shuttering (Papa) + ₹1.2L engineer, food, electrician, electrical items, vegetables
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Project_Home_Tracker.xlsx
+++ b/data/Project_Home_Tracker.xlsx
@@ -2759,7 +2759,7 @@
     <row r="12" ht="15.75" customHeight="1" s="99">
       <c r="A12" s="77" t="inlineStr">
         <is>
-          <t>Khutauna Chirai mill</t>
+          <t>Local Purchase</t>
         </is>
       </c>
       <c r="B12" s="87">
@@ -2789,7 +2789,7 @@
     <row r="13" ht="15.75" customHeight="1" s="99">
       <c r="A13" s="77" t="inlineStr">
         <is>
-          <t>Local Purchase</t>
+          <t>Khutauna Chirai mill</t>
         </is>
       </c>
       <c r="B13" s="87">
@@ -2849,7 +2849,7 @@
     <row r="15" ht="15.75" customHeight="1" s="99">
       <c r="A15" s="77" t="inlineStr">
         <is>
-          <t>Naveen Hardware</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B15" s="87">
@@ -2879,7 +2879,7 @@
     <row r="16" ht="15.75" customHeight="1" s="99">
       <c r="A16" s="77" t="inlineStr">
         <is>
-          <t>Sonbhai-Coordinator</t>
+          <t>Naveen Hardware</t>
         </is>
       </c>
       <c r="B16" s="87">
@@ -2909,50 +2909,88 @@
     <row r="17" ht="15.75" customHeight="1" s="99">
       <c r="A17" s="77" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>Subhash</t>
         </is>
       </c>
       <c r="B17" s="87">
-        <f>SUM(B5:B16)</f>
+        <f>COUNTIF('All Transactions'!H:H,A17)</f>
         <v/>
       </c>
       <c r="C17" s="87">
-        <f>SUM(C5:C16)</f>
+        <f>SUMIF('All Transactions'!H:H,A17,'All Transactions'!O:O)</f>
         <v/>
       </c>
       <c r="D17" s="87">
-        <f>SUM(D5:D16)</f>
+        <f>SUMIF('Payment Tracker'!D:D,A17,'Payment Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E17" s="97">
         <f>C17-D17</f>
         <v/>
       </c>
-      <c r="F17" s="89" t="n"/>
+      <c r="F17" s="89">
+        <f>IF(E17&gt;0,"⚠️ DUE",IF(E17&lt;0,"🔵 ADV","✅ PAID"))</f>
+        <v/>
+      </c>
       <c r="G17" s="90" t="n"/>
       <c r="H17" s="77" t="n"/>
       <c r="I17" s="82" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="99">
-      <c r="A18" s="82" t="n"/>
-      <c r="B18" s="82" t="n"/>
-      <c r="C18" s="82" t="n"/>
-      <c r="D18" s="82" t="n"/>
-      <c r="E18" s="82" t="n"/>
-      <c r="F18" s="82" t="n"/>
-      <c r="G18" s="82" t="n"/>
-      <c r="H18" s="82" t="n"/>
+      <c r="A18" s="77" t="inlineStr">
+        <is>
+          <t>Sonbhai-Coordinator</t>
+        </is>
+      </c>
+      <c r="B18" s="87">
+        <f>COUNTIF('All Transactions'!H:H,A18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="87">
+        <f>SUMIF('All Transactions'!H:H,A18,'All Transactions'!O:O)</f>
+        <v/>
+      </c>
+      <c r="D18" s="87">
+        <f>SUMIF('Payment Tracker'!D:D,A18,'Payment Tracker'!G:G)</f>
+        <v/>
+      </c>
+      <c r="E18" s="97">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="89">
+        <f>IF(E18&gt;0,"⚠️ DUE",IF(E18&lt;0,"🔵 ADV","✅ PAID"))</f>
+        <v/>
+      </c>
+      <c r="G18" s="90" t="n"/>
+      <c r="H18" s="77" t="n"/>
       <c r="I18" s="82" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="99">
-      <c r="A19" s="82" t="n"/>
-      <c r="B19" s="82" t="n"/>
-      <c r="C19" s="82" t="n"/>
-      <c r="D19" s="82" t="n"/>
-      <c r="E19" s="82" t="n"/>
-      <c r="F19" s="82" t="n"/>
-      <c r="G19" s="82" t="n"/>
-      <c r="H19" s="82" t="n"/>
+      <c r="A19" s="77" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="87">
+        <f>SUM(B5:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="87">
+        <f>SUM(C5:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="87">
+        <f>SUM(D5:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="97">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="89" t="n"/>
+      <c r="G19" s="90" t="n"/>
+      <c r="H19" s="77" t="n"/>
       <c r="I19" s="82" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="99">
@@ -3234,13 +3272,13 @@
       <c r="F7" s="113" t="n"/>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="120">
-        <f>-SUMIF('Vendor Summary'!E5:E16,"&lt;0")</f>
+        <f>-SUMIF('Vendor Summary'!E5:E18,"&lt;0")</f>
         <v/>
       </c>
       <c r="I7" s="113" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="121">
-        <f>SUMIF('Vendor Summary'!E5:E16,"&gt;0")</f>
+        <f>SUMIF('Vendor Summary'!E5:E18,"&gt;0")</f>
         <v/>
       </c>
       <c r="L7" s="113" t="n"/>
@@ -3755,11 +3793,11 @@
         </is>
       </c>
       <c r="I21" s="20">
-        <f>'Vendor Summary'!C17-SUM(I12:I20)</f>
+        <f>'Vendor Summary'!C19-SUM(I12:I20)</f>
         <v/>
       </c>
       <c r="J21" s="20">
-        <f>'Vendor Summary'!D17-SUM(J12:J20)</f>
+        <f>'Vendor Summary'!D19-SUM(J12:J20)</f>
         <v/>
       </c>
       <c r="K21" s="20">
@@ -6622,7 +6660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R659"/>
+  <dimension ref="A1:R665"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="99" min="1" max="1"/>
@@ -33800,33 +33838,393 @@
       </c>
     </row>
     <row r="659">
-      <c r="A659" s="60" t="inlineStr">
+      <c r="A659" t="n">
+        <v>667</v>
+      </c>
+      <c r="B659" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C659">
+        <f>IF(B659="","",TEXT(B659,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Shuttering Labour</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>Shuttering payment (Papa)</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I659" t="n">
+        <v>1</v>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K659" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L659">
+        <f>IF(OR(I659="",K659=""),"",I659*K659)</f>
+        <v/>
+      </c>
+      <c r="N659">
+        <f>M659*L659</f>
+        <v/>
+      </c>
+      <c r="O659">
+        <f>IF(L659="","",IF(M659="",L659,L659*(1-M659)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>668</v>
+      </c>
+      <c r="B660" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C660">
+        <f>IF(B660="","",TEXT(B660,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>Engineer payment</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="I660" t="n">
+        <v>1</v>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K660" t="n">
+        <v>120000</v>
+      </c>
+      <c r="L660">
+        <f>IF(OR(I660="",K660=""),"",I660*K660)</f>
+        <v/>
+      </c>
+      <c r="N660">
+        <f>M660*L660</f>
+        <v/>
+      </c>
+      <c r="O660">
+        <f>IF(L660="","",IF(M660="",L660,L660*(1-M660)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="n">
+        <v>669</v>
+      </c>
+      <c r="B661" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C661">
+        <f>IF(B661="","",TEXT(B661,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Food/Ration</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>Subhash — food</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>Subhash</t>
+        </is>
+      </c>
+      <c r="I661" t="n">
+        <v>1</v>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K661" t="n">
+        <v>3100</v>
+      </c>
+      <c r="L661">
+        <f>IF(OR(I661="",K661=""),"",I661*K661)</f>
+        <v/>
+      </c>
+      <c r="N661">
+        <f>M661*L661</f>
+        <v/>
+      </c>
+      <c r="O661">
+        <f>IF(L661="","",IF(M661="",L661,L661*(1-M661)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>670</v>
+      </c>
+      <c r="B662" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C662">
+        <f>IF(B662="","",TEXT(B662,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Electrician Labour</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>Electrician payment</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="I662" t="n">
+        <v>1</v>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K662" t="n">
+        <v>20000</v>
+      </c>
+      <c r="L662">
+        <f>IF(OR(I662="",K662=""),"",I662*K662)</f>
+        <v/>
+      </c>
+      <c r="N662">
+        <f>M662*L662</f>
+        <v/>
+      </c>
+      <c r="O662">
+        <f>IF(L662="","",IF(M662="",L662,L662*(1-M662)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>671</v>
+      </c>
+      <c r="B663" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C663">
+        <f>IF(B663="","",TEXT(B663,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Electrical Items</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>Electric pipe and concealed accessories</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I663" t="n">
+        <v>1</v>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K663" t="n">
+        <v>6800</v>
+      </c>
+      <c r="L663">
+        <f>IF(OR(I663="",K663=""),"",I663*K663)</f>
+        <v/>
+      </c>
+      <c r="N663">
+        <f>M663*L663</f>
+        <v/>
+      </c>
+      <c r="O663">
+        <f>IF(L663="","",IF(M663="",L663,L663*(1-M663)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="n">
+        <v>672</v>
+      </c>
+      <c r="B664" s="128" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C664">
+        <f>IF(B664="","",TEXT(B664,"MMM-YYYY"))</f>
+        <v/>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Plinth Phase</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Food/Ration</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="I664" t="n">
+        <v>1</v>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>Lumpsum</t>
+        </is>
+      </c>
+      <c r="K664" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L664">
+        <f>IF(OR(I664="",K664=""),"",I664*K664)</f>
+        <v/>
+      </c>
+      <c r="N664">
+        <f>M664*L664</f>
+        <v/>
+      </c>
+      <c r="O664">
+        <f>IF(L664="","",IF(M664="",L664,L664*(1-M664)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="60" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="B659" s="60" t="n"/>
-      <c r="C659" s="60" t="n"/>
-      <c r="D659" s="60" t="n"/>
-      <c r="E659" s="60" t="n"/>
-      <c r="F659" s="60" t="n"/>
-      <c r="G659" s="60" t="n"/>
-      <c r="H659" s="60" t="n"/>
-      <c r="I659" s="60" t="n"/>
-      <c r="J659" s="60" t="n"/>
-      <c r="K659" s="60" t="n"/>
-      <c r="L659" s="61">
-        <f>SUM(L5:L658)</f>
-        <v/>
-      </c>
-      <c r="M659" s="60" t="n"/>
-      <c r="N659" s="60" t="n"/>
-      <c r="O659" s="61">
+      <c r="B665" s="60" t="n"/>
+      <c r="C665" s="60" t="n"/>
+      <c r="D665" s="60" t="n"/>
+      <c r="E665" s="60" t="n"/>
+      <c r="F665" s="60" t="n"/>
+      <c r="G665" s="60" t="n"/>
+      <c r="H665" s="60" t="n"/>
+      <c r="I665" s="60" t="n"/>
+      <c r="J665" s="60" t="n"/>
+      <c r="K665" s="60" t="n"/>
+      <c r="L665" s="61">
+        <f>SUM(L5:L664)</f>
+        <v/>
+      </c>
+      <c r="M665" s="60" t="n"/>
+      <c r="N665" s="60" t="n"/>
+      <c r="O665" s="61">
         <f>SUM(O5:O528)</f>
         <v/>
       </c>
-      <c r="P659" s="60" t="n"/>
-      <c r="Q659" s="60" t="n"/>
+      <c r="P665" s="60" t="n"/>
+      <c r="Q665" s="60" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q504"/>
@@ -50925,16 +51323,44 @@
       <c r="A112" s="43" t="n">
         <v>118</v>
       </c>
-      <c r="B112" s="53" t="n"/>
-      <c r="C112" s="55" t="n"/>
-      <c r="D112" s="55" t="n"/>
-      <c r="E112" s="55" t="n"/>
-      <c r="F112" s="55" t="n"/>
-      <c r="G112" s="63" t="n"/>
-      <c r="H112" s="55" t="n"/>
+      <c r="B112" s="53" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C112" s="55" t="inlineStr">
+        <is>
+          <t>Papa</t>
+        </is>
+      </c>
+      <c r="D112" s="55" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E112" s="55" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F112" s="55" t="inlineStr">
+        <is>
+          <t>Shuttering payment (Papa)</t>
+        </is>
+      </c>
+      <c r="G112" s="63" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H112" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I112" s="55" t="n"/>
       <c r="J112" s="55" t="n"/>
-      <c r="K112" s="55" t="n"/>
+      <c r="K112" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L112" s="58">
         <f>IF(G112="","",IF(L111="",G112,L111+G112))</f>
         <v/>
@@ -50945,16 +51371,44 @@
       <c r="A113" s="41" t="n">
         <v>119</v>
       </c>
-      <c r="B113" s="45" t="n"/>
-      <c r="C113" s="47" t="n"/>
-      <c r="D113" s="47" t="n"/>
-      <c r="E113" s="47" t="n"/>
-      <c r="F113" s="47" t="n"/>
-      <c r="G113" s="62" t="n"/>
-      <c r="H113" s="47" t="n"/>
+      <c r="B113" s="45" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C113" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D113" s="47" t="inlineStr">
+        <is>
+          <t>Econ Builder</t>
+        </is>
+      </c>
+      <c r="E113" s="47" t="inlineStr">
+        <is>
+          <t>Professional Fees</t>
+        </is>
+      </c>
+      <c r="F113" s="47" t="inlineStr">
+        <is>
+          <t>Engineer payment</t>
+        </is>
+      </c>
+      <c r="G113" s="62" t="n">
+        <v>120000</v>
+      </c>
+      <c r="H113" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I113" s="47" t="n"/>
       <c r="J113" s="47" t="n"/>
-      <c r="K113" s="47" t="n"/>
+      <c r="K113" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L113" s="50">
         <f>IF(G113="","",IF(L112="",G113,L112+G113))</f>
         <v/>
@@ -50965,16 +51419,44 @@
       <c r="A114" s="43" t="n">
         <v>120</v>
       </c>
-      <c r="B114" s="53" t="n"/>
-      <c r="C114" s="55" t="n"/>
-      <c r="D114" s="55" t="n"/>
-      <c r="E114" s="55" t="n"/>
-      <c r="F114" s="55" t="n"/>
-      <c r="G114" s="63" t="n"/>
-      <c r="H114" s="55" t="n"/>
+      <c r="B114" s="53" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C114" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D114" s="55" t="inlineStr">
+        <is>
+          <t>Subhash</t>
+        </is>
+      </c>
+      <c r="E114" s="55" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F114" s="55" t="inlineStr">
+        <is>
+          <t>Subhash — food</t>
+        </is>
+      </c>
+      <c r="G114" s="63" t="n">
+        <v>3100</v>
+      </c>
+      <c r="H114" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I114" s="55" t="n"/>
       <c r="J114" s="55" t="n"/>
-      <c r="K114" s="55" t="n"/>
+      <c r="K114" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L114" s="58">
         <f>IF(G114="","",IF(L113="",G114,L113+G114))</f>
         <v/>
@@ -50985,16 +51467,44 @@
       <c r="A115" s="41" t="n">
         <v>121</v>
       </c>
-      <c r="B115" s="45" t="n"/>
-      <c r="C115" s="47" t="n"/>
-      <c r="D115" s="47" t="n"/>
-      <c r="E115" s="47" t="n"/>
-      <c r="F115" s="47" t="n"/>
-      <c r="G115" s="62" t="n"/>
-      <c r="H115" s="47" t="n"/>
+      <c r="B115" s="45" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C115" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D115" s="47" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="E115" s="47" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F115" s="47" t="inlineStr">
+        <is>
+          <t>Electrician payment</t>
+        </is>
+      </c>
+      <c r="G115" s="62" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H115" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I115" s="47" t="n"/>
       <c r="J115" s="47" t="n"/>
-      <c r="K115" s="47" t="n"/>
+      <c r="K115" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L115" s="50">
         <f>IF(G115="","",IF(L114="",G115,L114+G115))</f>
         <v/>
@@ -51005,16 +51515,44 @@
       <c r="A116" s="43" t="n">
         <v>122</v>
       </c>
-      <c r="B116" s="53" t="n"/>
-      <c r="C116" s="55" t="n"/>
-      <c r="D116" s="55" t="n"/>
-      <c r="E116" s="55" t="n"/>
-      <c r="F116" s="55" t="n"/>
-      <c r="G116" s="63" t="n"/>
-      <c r="H116" s="55" t="n"/>
+      <c r="B116" s="53" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C116" s="55" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D116" s="55" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="E116" s="55" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="F116" s="55" t="inlineStr">
+        <is>
+          <t>Electric pipe and concealed accessories</t>
+        </is>
+      </c>
+      <c r="G116" s="63" t="n">
+        <v>6800</v>
+      </c>
+      <c r="H116" s="55" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I116" s="55" t="n"/>
       <c r="J116" s="55" t="n"/>
-      <c r="K116" s="55" t="n"/>
+      <c r="K116" s="55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L116" s="58">
         <f>IF(G116="","",IF(L115="",G116,L115+G116))</f>
         <v/>
@@ -51025,16 +51563,44 @@
       <c r="A117" s="41" t="n">
         <v>123</v>
       </c>
-      <c r="B117" s="45" t="n"/>
-      <c r="C117" s="47" t="n"/>
-      <c r="D117" s="47" t="n"/>
-      <c r="E117" s="47" t="n"/>
-      <c r="F117" s="47" t="n"/>
-      <c r="G117" s="62" t="n"/>
-      <c r="H117" s="47" t="n"/>
+      <c r="B117" s="45" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C117" s="47" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="D117" s="47" t="inlineStr">
+        <is>
+          <t>Local Purchase</t>
+        </is>
+      </c>
+      <c r="E117" s="47" t="inlineStr">
+        <is>
+          <t>Transport · Food · Misc</t>
+        </is>
+      </c>
+      <c r="F117" s="47" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="G117" s="62" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H117" s="47" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
       <c r="I117" s="47" t="n"/>
       <c r="J117" s="47" t="n"/>
-      <c r="K117" s="47" t="n"/>
+      <c r="K117" s="47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L117" s="50">
         <f>IF(G117="","",IF(L116="",G117,L116+G117))</f>
         <v/>

</xml_diff>